<commit_message>
Set existing ground to ±0.00 and BOQ fill to 0.30 m
Owner confirmed the existing ground is at the road-around-building level
(±0.00); -1.50 is the public road. Fill for BOQ is 0.30 m over 64x58 m
= 1,113.60 m3, field density tests 16 points, fill task shortened to
6 days (handover 19 May 2027).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
+++ b/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
@@ -1446,7 +1446,7 @@
       <c r="J17" s="18" t="inlineStr"/>
       <c r="K17" s="19" t="inlineStr">
         <is>
-          <t>แผน CPM งานหลัก 5.4 เดือน (14 ธ.ค. 69 – 27 พ.ค. 70)</t>
+          <t>แผน CPM งานหลัก 5.2 เดือน (14 ธ.ค. 69 – 19 พ.ค. 70)</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="C20" s="24" t="n">
-        <v>8566</v>
+        <v>1113.6</v>
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="K20" s="19" t="inlineStr">
         <is>
-          <t>เดิม 1,856 (ถมเฉลี่ย 0.50 ม.) → A202: ถนนอ้างอิง -1.50 / ถนนรอบอาคาร ±0.00 / FFL +0.50 ถ้าดินเดิม -1.50 = 8,566; -1.00 = 5,593; -0.50 = 2,620 ลบ.ม. ยืนยันด้วยผลสำรวจระดับ P1.2 และเสนอราคาต่อ ลบ.ม.</t>
+          <t>เดิม 1,856 (ถม 0.50 ม.) → ผู้ว่าจ้างกำหนด: ดินเดิม ±0.00 (ระดับถนนรอบอาคาร; -1.50 คือถนนสาธารณะ) ถมหนา 0.30 ม. x 64 x 58 ม. = 1,113.60 ลบ.ม. เบิกตามปริมาณจริงจากผลสำรวจระดับ P1.2</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B24" s="26" t="inlineStr">
         <is>
-          <t>ป้องกันดินพังและสูบน้ำ งานขุดถังเก็บน้ำใต้ดิน ลึก ~3.0 ม. (Sheet pile/ค้ำยัน)</t>
+          <t>ป้องกันดินพังและสูบน้ำ งานขุดถังเก็บน้ำใต้ดิน ลึก ~3.0 ม. จากดินเดิม ±0.00 (Sheet pile/ค้ำยัน)</t>
         </is>
       </c>
       <c r="C24" s="27" t="n">
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="C28" s="24" t="n">
-        <v>96</v>
+        <v>16</v>
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="K28" s="19" t="inlineStr">
         <is>
-          <t>เดิม 6 → พื้นที่ 5,946 ตร.ม. ÷ 500 = 12 จุด/ชั้น x 8 ชั้น (ถม 1.60 ม. ชั้นละ 0.20)</t>
+          <t>เดิม 6 → พื้นที่ถม 3,712 ตร.ม. ÷ 500 = 8 จุด/ชั้น x 2 ชั้น (ถม 0.30 ม. ชั้นละไม่เกิน 0.20)</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="D6" s="37" t="inlineStr">
         <is>
-          <t>เดิม 1,856 (ถมเฉลี่ย 0.50 ม.) → A202: ถนนอ้างอิง -1.50 / ถนนรอบอาคาร ±0.00 / FFL +0.50 ถ้าดินเดิม -1.50 = 8,566; -1.00 = 5,593; -0.50 = 2,620 ลบ.ม. ยืนยันด้วยผลสำรวจระดับ P1.2 และเสนอราคาต่อ ลบ.ม.</t>
+          <t>เดิม 1,856 (ถม 0.50 ม.) → ผู้ว่าจ้างกำหนด: ดินเดิม ±0.00 (ระดับถนนรอบอาคาร; -1.50 คือถนนสาธารณะ) ถมหนา 0.30 ม. x 64 x 58 ม. = 1,113.60 ลบ.ม. เบิกตามปริมาณจริงจากผลสำรวจระดับ P1.2</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="C8" s="37" t="inlineStr">
         <is>
-          <t>ป้องกันดินพังและสูบน้ำ งานขุดถังเก็บน้ำใต้ดิน ลึก ~3.0 ม. (Sheet pile/ค้ำยัน)</t>
+          <t>ป้องกันดินพังและสูบน้ำ งานขุดถังเก็บน้ำใต้ดิน ลึก ~3.0 ม. จากดินเดิม ±0.00 (Sheet pile/ค้ำยัน)</t>
         </is>
       </c>
       <c r="D8" s="37" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="D10" s="37" t="inlineStr">
         <is>
-          <t>เดิม 6 → พื้นที่ 5,946 ตร.ม. ÷ 500 = 12 จุด/ชั้น x 8 ชั้น (ถม 1.60 ม. ชั้นละ 0.20)</t>
+          <t>เดิม 6 → พื้นที่ถม 3,712 ตร.ม. ÷ 500 = 8 จุด/ชั้น x 2 ชั้น (ถม 0.30 ม. ชั้นละไม่เกิน 0.20)</t>
         </is>
       </c>
     </row>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C75" s="37" t="inlineStr">
         <is>
-          <t>ปริมาณดินถมขึ้นกับระดับดินเดิม ต้องยืนยันด้วยสำรวจระดับ P1.2 แนะนำเสนอเป็นราคาต่อ ลบ.ม. และคิดตามปริมาณจริง</t>
+          <t>ผู้ว่าจ้างยืนยัน 27/10/69: ดินเดิมอยู่ที่ ±0.00 (ระดับถนนรอบอาคาร) ระดับ -1.50 คือถนนสาธารณะ คิด BOQ ถมหนา 0.30 ม. ปริมาณจริงเบิกตามผลสำรวจระดับ P1.2</t>
         </is>
       </c>
       <c r="D75" s="37" t="inlineStr"/>

</xml_diff>

<commit_message>
Split piles into building, annex/other and road groups
- separate layers and 4D tasks: building piles 452 (M21A), annex/other
  50 (M21B: F1P-1, tank, transformer, boundary pads), road 249 (M21C)
- road piles 249 confirmed for BOQ; drawings show 232 positions, the
  remaining 17 are reported, not placed
- annex F1P-1 footings moved to the annex task after their piles
- north side (grid A) confirmed; temporary office, store and toilets
  moved to the north strip between road pile rows, road slab under them
  cast after removal
- stage highlight tints each layer colour instead of replacing it

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
+++ b/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
@@ -1288,20 +1288,20 @@
       <c r="K11" s="19" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>1.2.3</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>สำนักงานสนาม (Site Office) ขนาดไม่น้อยกว่า 3.00 x 8.00 ม. พร้อมเครื่องปรับอากาศ โต๊ะประชุม และอุปกรณ์สำนักงาน</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>หลัง</t>
         </is>
@@ -1320,10 +1320,14 @@
         <f>F12+H12</f>
         <v/>
       </c>
-      <c r="J12" s="18" t="inlineStr"/>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
+        </is>
+      </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
-          <t>รวมพื้นที่สำหรับผู้ควบคุมงานของผู้ว่าจ้าง</t>
+          <t>รวมพื้นที่สำหรับผู้ควบคุมงานของผู้ว่าจ้าง; วางด้านทิศเหนือของอาคาร แนวกริด 1-2</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1371,7 @@
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>พื้นที่ว่างรอบอาคารแคบ (4-14 ม.) ต้องย้ายออกก่อนงานพื้นถนน หรือเช่าพื้นที่ข้างเคียง</t>
+          <t>วางด้านทิศเหนือระหว่างแถวเข็มถนน (ผู้ว่าจ้างกำหนด) ขนาด 3.00x12.00 ม.; พื้นถนนใต้สิ่งชั่วคราวเทหลังรื้อย้าย</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2492,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>หมวดงานเสาเข็ม (ตอกรูปตัวไอ ยาว 22 ม. ตาม Type Mark ปรับความยาวตามผลสำรวจดิน P3)</t>
+          <t>หมวดงานเสาเข็ม (กลุ่มเข็มอาคาร 2.1.1-2.1.2 / กลุ่มเข็มอาคารประกอบ-อื่นๆ 2.1.3-2.1.4, 4.3.1, 4.6.1 / กลุ่มเข็มถนน 4.1.1) ยาว 22 ม.</t>
         </is>
       </c>
       <c r="C5" s="17" t="n"/>
@@ -2713,7 +2717,7 @@
       </c>
       <c r="K10" s="19" t="inlineStr">
         <is>
-          <t>เดิม 470 → รวมทุกชนิดในหมวด 2.1 + 4.1 + 4.3 + 4.6</t>
+          <t>เดิม 470 → 3 กลุ่ม: อาคาร 452 + อาคารประกอบ/อื่นๆ 50 + ถนน 249 = 751</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5563,7 @@
       </c>
       <c r="K6" s="19" t="inlineStr">
         <is>
-          <t>ตาราง S2 = 249; นับจากผัง S201 ได้ 232 (ยืนยันจำนวน)</t>
+          <t>กลุ่มเข็มถนน: ผู้ว่าจ้างยืนยัน 249 ต้น (ผัง S201/S202 แสดงตำแหน่ง 232 ต้น ขอตำแหน่งอีก 17 ต้นจากผู้ออกแบบ)</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5607,7 @@
       </c>
       <c r="K7" s="19" t="inlineStr">
         <is>
-          <t>คอนกรีต 26.78, ทราย 35.86, คอนกรีตหยาบ 6.10 ลบ.ม. (S1.1)</t>
+          <t>ตามเข็มถนน 249 ต้น คอนกรีต 26.78, ทราย 35.86, คอนกรีตหยาบ 6.10 ลบ.ม. (S1.1)</t>
         </is>
       </c>
     </row>
@@ -6873,7 +6877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6980,7 +6984,7 @@
     <row r="6">
       <c r="A6" s="37" t="inlineStr">
         <is>
-          <t>1.2.4</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B6" s="38" t="inlineStr">
@@ -6990,19 +6994,19 @@
       </c>
       <c r="C6" s="37" t="inlineStr">
         <is>
-          <t>โรงเก็บวัสดุและเครื่องมือ (Store) พร้อมลานกองเหล็กเสริมและลานดัดเหล็ก</t>
+          <t>สำนักงานสนาม (Site Office) ขนาดไม่น้อยกว่า 3.00 x 8.00 ม. พร้อมเครื่องปรับอากาศ โต๊ะประชุม และอุปกรณ์สำนักงาน</t>
         </is>
       </c>
       <c r="D6" s="37" t="inlineStr">
         <is>
-          <t>พื้นที่ว่างรอบอาคารแคบ (4-14 ม.) ต้องย้ายออกก่อนงานพื้นถนน หรือเช่าพื้นที่ข้างเคียง</t>
+          <t>รวมพื้นที่สำหรับผู้ควบคุมงานของผู้ว่าจ้าง; วางด้านทิศเหนือของอาคาร แนวกริด 1-2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="37" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="B7" s="38" t="inlineStr">
@@ -7012,41 +7016,41 @@
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
-          <t>ถมดินปรับระดับ บดอัดเป็นชั้นหนาไม่เกิน 0.20 ม. ความแน่นไม่น้อยกว่า 95% Standard Proctor</t>
+          <t>โรงเก็บวัสดุและเครื่องมือ (Store) พร้อมลานกองเหล็กเสริมและลานดัดเหล็ก</t>
         </is>
       </c>
       <c r="D7" s="37" t="inlineStr">
         <is>
-          <t>เดิม 1,856 (ถม 0.50 ม.) → ผู้ว่าจ้างกำหนด: ดินเดิม ±0.00 (ระดับถนนรอบอาคาร; -1.50 คือถนนสาธารณะ) ถมหนา 0.30 ม. x 64 x 58 ม. = 1,113.60 ลบ.ม. เบิกตามปริมาณจริงจากผลสำรวจระดับ P1.2</t>
+          <t>วางด้านทิศเหนือระหว่างแถวเข็มถนน (ผู้ว่าจ้างกำหนด) ขนาด 3.00x12.00 ม.; พื้นถนนใต้สิ่งชั่วคราวเทหลังรื้อย้าย</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="37" t="inlineStr">
         <is>
-          <t>1.3.4</t>
-        </is>
-      </c>
-      <c r="B8" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C8" s="37" t="inlineStr">
         <is>
-          <t>ขุดดินฐานรากและขนย้ายดินส่วนเกิน (จากตาราง S1.1)</t>
+          <t>ถมดินปรับระดับ บดอัดเป็นชั้นหนาไม่เกิน 0.20 ม. ความแน่นไม่น้อยกว่า 95% Standard Proctor</t>
         </is>
       </c>
       <c r="D8" s="37" t="inlineStr">
         <is>
-          <t>S201-B ตาราง S1.1 รวม F1/F1A/F1P/F2P (ไม่รวมถังใต้ดิน 4.4)</t>
+          <t>เดิม 1,856 (ถม 0.50 ม.) → ผู้ว่าจ้างกำหนด: ดินเดิม ±0.00 (ระดับถนนรอบอาคาร; -1.50 คือถนนสาธารณะ) ถมหนา 0.30 ม. x 64 x 58 ม. = 1,113.60 ลบ.ม. เบิกตามปริมาณจริงจากผลสำรวจระดับ P1.2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="37" t="inlineStr">
         <is>
-          <t>1.3.5</t>
+          <t>1.3.4</t>
         </is>
       </c>
       <c r="B9" s="39" t="inlineStr">
@@ -7056,19 +7060,19 @@
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
-          <t>ป้องกันดินพังและสูบน้ำ งานขุดถังเก็บน้ำใต้ดิน ลึก ~3.0 ม. จากดินเดิม ±0.00 (Sheet pile/ค้ำยัน)</t>
+          <t>ขุดดินฐานรากและขนย้ายดินส่วนเกิน (จากตาราง S1.1)</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
         <is>
-          <t>ระดับก้นถัง BF -2.85 (S202)</t>
+          <t>S201-B ตาราง S1.1 รวม F1/F1A/F1P/F2P (ไม่รวมถังใต้ดิน 4.4)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="37" t="inlineStr">
         <is>
-          <t>1.3.6</t>
+          <t>1.3.5</t>
         </is>
       </c>
       <c r="B10" s="39" t="inlineStr">
@@ -7078,41 +7082,41 @@
       </c>
       <c r="C10" s="37" t="inlineStr">
         <is>
-          <t>ถมดินกลับรอบฐานราก บดอัด (จากตาราง S1.1)</t>
+          <t>ป้องกันดินพังและสูบน้ำ งานขุดถังเก็บน้ำใต้ดิน ลึก ~3.0 ม. จากดินเดิม ±0.00 (Sheet pile/ค้ำยัน)</t>
         </is>
       </c>
       <c r="D10" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: S201-B ตาราง S1.1 คอลัมน์ดินถม</t>
+          <t>ระดับก้นถัง BF -2.85 (S202)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="37" t="inlineStr">
         <is>
-          <t>1.4.2</t>
-        </is>
-      </c>
-      <c r="B11" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>1.3.6</t>
+        </is>
+      </c>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
-          <t>ทดสอบกำลังรับน้ำหนักเสาเข็มแบบพลศาสตร์ (Dynamic Load Test)</t>
+          <t>ถมดินกลับรอบฐานราก บดอัด (จากตาราง S1.1)</t>
         </is>
       </c>
       <c r="D11" s="37" t="inlineStr">
         <is>
-          <t>เดิม 2 → อย่างน้อย 1 ต้นต่อขนาดเข็ม (I22/I26/I35) หรือตามวิศวกรกำหนด</t>
+          <t>เพิ่ม: S201-B ตาราง S1.1 คอลัมน์ดินถม</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="37" t="inlineStr">
         <is>
-          <t>1.4.3</t>
+          <t>1.4.2</t>
         </is>
       </c>
       <c r="B12" s="38" t="inlineStr">
@@ -7122,19 +7126,19 @@
       </c>
       <c r="C12" s="37" t="inlineStr">
         <is>
-          <t>ทดสอบความแน่นดินถมในสนาม (Field Density Test)</t>
+          <t>ทดสอบกำลังรับน้ำหนักเสาเข็มแบบพลศาสตร์ (Dynamic Load Test)</t>
         </is>
       </c>
       <c r="D12" s="37" t="inlineStr">
         <is>
-          <t>เดิม 6 → พื้นที่ถม 3,712 ตร.ม. ÷ 500 = 8 จุด/ชั้น x 2 ชั้น (ถม 0.30 ม. ชั้นละไม่เกิน 0.20)</t>
+          <t>เดิม 2 → อย่างน้อย 1 ต้นต่อขนาดเข็ม (I22/I26/I35) หรือตามวิศวกรกำหนด</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="37" t="inlineStr">
         <is>
-          <t>1.4.4</t>
+          <t>1.4.3</t>
         </is>
       </c>
       <c r="B13" s="38" t="inlineStr">
@@ -7144,63 +7148,63 @@
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
-          <t>ทดสอบวัสดุก่อสร้าง (ตัวอย่างคอนกรีต กำลังดึงเหล็กเสริม) ตลอดโครงการ</t>
+          <t>ทดสอบความแน่นดินถมในสนาม (Field Density Test)</t>
         </is>
       </c>
       <c r="D13" s="37" t="inlineStr">
         <is>
-          <t>คอนกรีตโครงสร้างรวม ~1,270 ลบ.ม. (ไม่รวมถังใต้ดิน/ทางลาด)</t>
+          <t>เดิม 6 → พื้นที่ถม 3,712 ตร.ม. ÷ 500 = 8 จุด/ชั้น x 2 ชั้น (ถม 0.30 ม. ชั้นละไม่เกิน 0.20)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="37" t="inlineStr">
         <is>
-          <t>1.4.5</t>
-        </is>
-      </c>
-      <c r="B14" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>1.4.4</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C14" s="37" t="inlineStr">
         <is>
-          <t>เครนยกติดตั้ง รถกระเช้า (Man lift) และนั่งร้านงานสูง +9.00 ถึง +15.25 ม.</t>
+          <t>ทดสอบวัสดุก่อสร้าง (ตัวอย่างคอนกรีต กำลังดึงเหล็กเสริม) ตลอดโครงการ</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: งานโครงเหล็ก/หลังคา/Jack roof (A202)</t>
+          <t>คอนกรีตโครงสร้างรวม ~1,270 ลบ.ม. (ไม่รวมถังใต้ดิน/ทางลาด)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="37" t="inlineStr">
         <is>
-          <t>2.1.2</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>1.4.5</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-350x350 ยาว 22 ม. รับพื้นโรงงาน (I35-22) ระยะ 3.00x3.00 ม. รวมค่าตอก</t>
+          <t>เครนยกติดตั้ง รถกระเช้า (Man lift) และนั่งร้านงานสูง +9.00 ถึง +15.25 ม.</t>
         </is>
       </c>
       <c r="D15" s="37" t="inlineStr">
         <is>
-          <t>ตรงกัน 360 ต้น; ระบุขนาด 350 มม. (ราคาต่างจากเข็มฐานราก)</t>
+          <t>เพิ่ม: งานโครงเหล็ก/หลังคา/Jack roof (A202)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="37" t="inlineStr">
         <is>
-          <t>2.1.3</t>
+          <t>2.1.2</t>
         </is>
       </c>
       <c r="B16" s="38" t="inlineStr">
@@ -7210,85 +7214,85 @@
       </c>
       <c r="C16" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-260x260 ยาว 22 ม. อาคารประกอบ ฐาน F1P-1 (ห้องน้ำ 6, ห้องสารเคมี 3, ทางลาดเหนือ 2) รวมค่าตอก</t>
+          <t>เสาเข็มตอก I-350x350 ยาว 22 ม. รับพื้นโรงงาน (I35-22) ระยะ 3.00x3.00 ม. รวมค่าตอก</t>
         </is>
       </c>
       <c r="D16" s="37" t="inlineStr">
         <is>
-          <t>เดิม 18 → 11 (นับจาก S201)</t>
+          <t>ตรงกัน 360 ต้น; ระบุขนาด 350 มม. (ราคาต่างจากเข็มฐานราก)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="37" t="inlineStr">
         <is>
-          <t>2.1.4</t>
-        </is>
-      </c>
-      <c r="B17" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.1.3</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-260x260 รับถังเก็บน้ำใต้ดิน (ตัดหัวลดระดับ 1 ม.) รวมค่าตอก</t>
+          <t>เสาเข็มตอก I-260x260 ยาว 22 ม. อาคารประกอบ ฐาน F1P-1 (ห้องน้ำ 6, ห้องสารเคมี 3, ทางลาดเหนือ 2) รวมค่าตอก</t>
         </is>
       </c>
       <c r="D17" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: S201-B (I26) นับจากผังได้ 17</t>
+          <t>เดิม 18 → 11 (นับจาก S201)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="37" t="inlineStr">
         <is>
-          <t>2.1.5</t>
-        </is>
-      </c>
-      <c r="B18" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>2.1.4</t>
+        </is>
+      </c>
+      <c r="B18" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C18" s="37" t="inlineStr">
         <is>
-          <t>ตัดหัวเสาเข็มและขนทิ้ง</t>
+          <t>เสาเข็มตอก I-260x260 รับถังเก็บน้ำใต้ดิน (ตัดหัวลดระดับ 1 ม.) รวมค่าตอก</t>
         </is>
       </c>
       <c r="D18" s="37" t="inlineStr">
         <is>
-          <t>เดิม 470 → รวมทุกชนิดในหมวด 2.1 + 4.1 + 4.3 + 4.6</t>
+          <t>เพิ่ม: S201-B (I26) นับจากผังได้ 17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="37" t="inlineStr">
         <is>
-          <t>2.1.6</t>
-        </is>
-      </c>
-      <c r="B19" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.1.5</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
-          <t>ราคาปรับเพิ่ม/ลดความยาวเสาเข็ม กรณีผลสำรวจดินต่างจากความยาวที่สมมติ แยกตามขนาด I22 / I26 / I35</t>
+          <t>ตัดหัวเสาเข็มและขนทิ้ง</t>
         </is>
       </c>
       <c r="D19" s="37" t="inlineStr">
         <is>
-          <t>ราคาต่อเมตร (ไม่มีปริมาณ) ใช้ปรับหลังได้ผลสำรวจดิน P3</t>
+          <t>เดิม 470 → 3 กลุ่ม: อาคาร 452 + อาคารประกอบ/อื่นๆ 50 + ถนน 249 = 751</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="37" t="inlineStr">
         <is>
-          <t>2.1.7</t>
+          <t>2.1.6</t>
         </is>
       </c>
       <c r="B20" s="40" t="inlineStr">
@@ -7298,63 +7302,63 @@
       </c>
       <c r="C20" s="37" t="inlineStr">
         <is>
-          <t>เชื่อมต่อเสาเข็ม (เข็มยาว 22 ม. ส่ง 2 ท่อน) พร้อมแผ่นเหล็กต่อเชื่อม</t>
+          <t>ราคาปรับเพิ่ม/ลดความยาวเสาเข็ม กรณีผลสำรวจดินต่างจากความยาวที่สมมติ แยกตามขนาด I22 / I26 / I35</t>
         </is>
       </c>
       <c r="D20" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: สมมติ 1 รอยต่อ/ต้น ตามความยาวท่อนที่ผู้ผลิตส่งได้</t>
+          <t>ราคาต่อเมตร (ไม่มีปริมาณ) ใช้ปรับหลังได้ผลสำรวจดิน P3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="37" t="inlineStr">
         <is>
-          <t>2.2.1</t>
-        </is>
-      </c>
-      <c r="B21" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>2.1.7</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
-          <t>ฐานราก F2P 0.60x1.50x0.80 ม. (เข็ม 2 ต้น) ทรายรองพื้น คอนกรีตหยาบ คอนกรีตโครงสร้าง ไม้แบบ</t>
+          <t>เชื่อมต่อเสาเข็ม (เข็มยาว 22 ม. ส่ง 2 ท่อน) พร้อมแผ่นเหล็กต่อเชื่อม</t>
         </is>
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
-          <t>ผู้ว่าจ้างยืนยัน 46 ฐาน (เสา C1 45 + C2 1, เข็ม 2 ต้น/ฐาน = 92 ต้น) ตาราง S1.1 นับ 47 ผิด; คอนกรีต 33.12 ลบ.ม., ทราย 11.84, คอนกรีตหยาบ 2.63, ไม้แบบ 154.56 ตร.ม.</t>
+          <t>เพิ่ม: สมมติ 1 รอยต่อ/ต้น ตามความยาวท่อนที่ผู้ผลิตส่งได้</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="37" t="inlineStr">
         <is>
-          <t>2.2.2</t>
-        </is>
-      </c>
-      <c r="B22" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.2.1</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C22" s="37" t="inlineStr">
         <is>
-          <t>Drop panel F1P 1.00x1.00x0.20 ม. รับพื้นบนเข็ม I35 ทรายรองพื้น คอนกรีตหยาบ คอนกรีต</t>
+          <t>ฐานราก F2P 0.60x1.50x0.80 ม. (เข็ม 2 ต้น) ทรายรองพื้น คอนกรีตหยาบ คอนกรีตโครงสร้าง ไม้แบบ</t>
         </is>
       </c>
       <c r="D22" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: คอนกรีต 72.00, ทราย 92.16, คอนกรีตหยาบ 21.78 ลบ.ม.</t>
+          <t>ผู้ว่าจ้างยืนยัน 46 ฐาน (เสา C1 45 + C2 1, เข็ม 2 ต้น/ฐาน = 92 ต้น) ตาราง S1.1 นับ 47 ผิด; คอนกรีต 33.12 ลบ.ม., ทราย 11.84, คอนกรีตหยาบ 2.63, ไม้แบบ 154.56 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="37" t="inlineStr">
         <is>
-          <t>2.2.3</t>
+          <t>2.2.2</t>
         </is>
       </c>
       <c r="B23" s="39" t="inlineStr">
@@ -7364,85 +7368,85 @@
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
-          <t>ฐาน F1P-1 0.60x0.60x0.60 ม. (เข็มเดี่ยว อาคารประกอบ)</t>
+          <t>Drop panel F1P 1.00x1.00x0.20 ม. รับพื้นบนเข็ม I35 ทรายรองพื้น คอนกรีตหยาบ คอนกรีต</t>
         </is>
       </c>
       <c r="D23" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: คอนกรีต 2.38, ทราย 1.58, คอนกรีตหยาบ 0.27 ลบ.ม.</t>
+          <t>เพิ่ม: คอนกรีต 72.00, ทราย 92.16, คอนกรีตหยาบ 21.78 ลบ.ม.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="37" t="inlineStr">
         <is>
-          <t>2.2.4</t>
-        </is>
-      </c>
-      <c r="B24" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.2.3</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C24" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริมฐานราก F2P / F1P / F1P-1</t>
+          <t>ฐาน F1P-1 0.60x0.60x0.60 ม. (เข็มเดี่ยว อาคารประกอบ)</t>
         </is>
       </c>
       <c r="D24" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม (อ้างอิงประมาณ 100 กก./ลบ.ม. ≈ 10,750 กก.)</t>
+          <t>เพิ่ม: คอนกรีต 2.38, ทราย 1.58, คอนกรีตหยาบ 0.27 ลบ.ม.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="37" t="inlineStr">
         <is>
-          <t>2.3.1</t>
-        </is>
-      </c>
-      <c r="B25" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>2.2.4</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
-          <t>เสา คสล. C1 0.30x0.50 ม. จากหลังฐานรากถึงหัวเสา +4.50 (ยาว 4.90 ม.)</t>
+          <t>เหล็กเสริมฐานราก F2P / F1P / F1P-1</t>
         </is>
       </c>
       <c r="D25" s="37" t="inlineStr">
         <is>
-          <t>เดิม 'เสาตอม่อ 46' → C1 45 ต้น คอนกรีต 32.37 ลบ.ม. ไม้แบบ 352.80 ตร.ม. (S4.1)</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม (อ้างอิงประมาณ 100 กก./ลบ.ม. ≈ 10,750 กก.)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="37" t="inlineStr">
         <is>
-          <t>2.3.2</t>
-        </is>
-      </c>
-      <c r="B26" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.3.1</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
-          <t>เสา คสล. C2 0.50x0.50 ม. (กริด 6/J)</t>
+          <t>เสา คสล. C1 0.30x0.50 ม. จากหลังฐานรากถึงหัวเสา +4.50 (ยาว 4.90 ม.)</t>
         </is>
       </c>
       <c r="D26" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: คอนกรีต 1.13 ลบ.ม. ไม้แบบ 9.80 ตร.ม.</t>
+          <t>เดิม 'เสาตอม่อ 46' → C1 45 ต้น คอนกรีต 32.37 ลบ.ม. ไม้แบบ 352.80 ตร.ม. (S4.1)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="37" t="inlineStr">
         <is>
-          <t>2.3.3</t>
+          <t>2.3.2</t>
         </is>
       </c>
       <c r="B27" s="39" t="inlineStr">
@@ -7452,239 +7456,239 @@
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
-          <t>เสา คสล. C3 0.20x0.20 ม. อาคารประกอบ</t>
+          <t>เสา คสล. C2 0.50x0.50 ม. (กริด 6/J)</t>
         </is>
       </c>
       <c r="D27" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: คอนกรีต 1.60 ลบ.ม. ไม้แบบ 34.74 ตร.ม. (S4.1 รวม 3 ระดับ)</t>
+          <t>เพิ่ม: คอนกรีต 1.13 ลบ.ม. ไม้แบบ 9.80 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="37" t="inlineStr">
         <is>
-          <t>2.3.4</t>
-        </is>
-      </c>
-      <c r="B28" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>2.3.3</t>
+        </is>
+      </c>
+      <c r="B28" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C28" s="37" t="inlineStr">
         <is>
-          <t>คานคอดิน B1 0.20x0.60 ม. TOP +0.50 (แนวรอบอาคาร + แนวกริด 6)</t>
+          <t>เสา คสล. C3 0.20x0.20 ม. อาคารประกอบ</t>
         </is>
       </c>
       <c r="D28" s="37" t="inlineStr">
         <is>
-          <t>เดิมว่าง → คอนกรีต 32.04 ลบ.ม. ไม้แบบ 394.80 ตร.ม. (S3)</t>
+          <t>เพิ่ม: คอนกรีต 1.60 ลบ.ม. ไม้แบบ 34.74 ตร.ม. (S4.1 รวม 3 ระดับ)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="37" t="inlineStr">
         <is>
-          <t>2.3.5</t>
-        </is>
-      </c>
-      <c r="B29" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.3.4</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
-          <t>คาน B3 0.20x0.40 ม. อาคารประกอบ (ระดับถนน + ระดับพื้นชั้น 1)</t>
+          <t>คานคอดิน B1 0.20x0.60 ม. TOP +0.50 (แนวรอบอาคาร + แนวกริด 6)</t>
         </is>
       </c>
       <c r="D29" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: คอนกรีต 1.81 ลบ.ม. ไม้แบบ 40.45 ตร.ม. (S3)</t>
+          <t>เดิมว่าง → คอนกรีต 32.04 ลบ.ม. ไม้แบบ 394.80 ตร.ม. (S3)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="37" t="inlineStr">
         <is>
-          <t>2.3.6</t>
-        </is>
-      </c>
-      <c r="B30" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.3.5</t>
+        </is>
+      </c>
+      <c r="B30" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C30" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริมเสาและคาน คสล. (C1, C2, C3, B1, B3)</t>
+          <t>คาน B3 0.20x0.40 ม. อาคารประกอบ (ระดับถนน + ระดับพื้นชั้น 1)</t>
         </is>
       </c>
       <c r="D30" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม (อ้างอิงประมาณ 160 กก./ลบ.ม. ≈ 11,000 กก.)</t>
+          <t>เพิ่ม: คอนกรีต 1.81 ลบ.ม. ไม้แบบ 40.45 ตร.ม. (S3)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="37" t="inlineStr">
         <is>
-          <t>2.4.1</t>
-        </is>
-      </c>
-      <c r="B31" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>2.3.6</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
-          <t>พื้น S1 คสล. หนา 0.20 ม. วางบนเสาเข็ม TOP +0.50 พร้อมไม้แบบข้าง</t>
+          <t>เหล็กเสริมเสาและคาน คสล. (C1, C2, C3, B1, B3)</t>
         </is>
       </c>
       <c r="D31" s="37" t="inlineStr">
         <is>
-          <t>เดิม 3,240 → 3,206.48 ตร.ม. คอนกรีต 641.30 ลบ.ม. (S6.1)</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม (อ้างอิงประมาณ 160 กก./ลบ.ม. ≈ 11,000 กก.)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="37" t="inlineStr">
         <is>
-          <t>2.4.2</t>
-        </is>
-      </c>
-      <c r="B32" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.4.1</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C32" s="37" t="inlineStr">
         <is>
-          <t>พื้นห้อง SF02 หนา 0.25 / AF01 หนา 0.10 ระดับพื้นชั้น 1</t>
+          <t>พื้น S1 คสล. หนา 0.20 ม. วางบนเสาเข็ม TOP +0.50 พร้อมไม้แบบข้าง</t>
         </is>
       </c>
       <c r="D32" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: SF02 30.50 + AF01 21.32 ตร.ม. คอนกรีต 9.76 ลบ.ม. (S6.1)</t>
+          <t>เดิม 3,240 → 3,206.48 ตร.ม. คอนกรีต 641.30 ลบ.ม. (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="37" t="inlineStr">
         <is>
-          <t>2.4.3</t>
-        </is>
-      </c>
-      <c r="B33" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.4.2</t>
+        </is>
+      </c>
+      <c r="B33" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม/ตะแกรงเหล็ก พื้น S1, SF02, AF01</t>
+          <t>พื้นห้อง SF02 หนา 0.25 / AF01 หนา 0.10 ระดับพื้นชั้น 1</t>
         </is>
       </c>
       <c r="D33" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม (อ้างอิงประมาณ 80 กก./ลบ.ม. ≈ 52,000 กก.)</t>
+          <t>เพิ่ม: SF02 30.50 + AF01 21.32 ตร.ม. คอนกรีต 9.76 ลบ.ม. (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="37" t="inlineStr">
         <is>
-          <t>2.4.4</t>
-        </is>
-      </c>
-      <c r="B34" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.4.3</t>
+        </is>
+      </c>
+      <c r="B34" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C34" s="37" t="inlineStr">
         <is>
-          <t>แผ่นพลาสติก PE รองใต้พื้น S1 และทรายรองพื้น</t>
+          <t>เหล็กเสริม/ตะแกรงเหล็ก พื้น S1, SF02, AF01</t>
         </is>
       </c>
       <c r="D34" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: พื้นที่ S1 (S6.1)</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม (อ้างอิงประมาณ 80 กก./ลบ.ม. ≈ 52,000 กก.)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="37" t="inlineStr">
         <is>
-          <t>2.4.5</t>
-        </is>
-      </c>
-      <c r="B35" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.4.4</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
-          <t>ตัดรอยต่อพื้น (Saw cut) และยาแนว Joint sealant พื้น S1</t>
+          <t>แผ่นพลาสติก PE รองใต้พื้น S1 และทรายรองพื้น</t>
         </is>
       </c>
       <c r="D35" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: สมมติรอยต่อทุก 6 ม. ตามแนวกริด (9x54 + 8x60 ม.) รอแบบ</t>
+          <t>เพิ่ม: พื้นที่ S1 (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="37" t="inlineStr">
         <is>
-          <t>2.5.1</t>
-        </is>
-      </c>
-      <c r="B36" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>2.4.5</t>
+        </is>
+      </c>
+      <c r="B36" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C36" s="37" t="inlineStr">
         <is>
-          <t>เสาเหล็ก H250x175x44.1 กก./ม. บนหัวเสา คสล. +4.50 ถึง +9.00 พร้อมแผ่นเหล็กฐาน Anchor bolt</t>
+          <t>ตัดรอยต่อพื้น (Saw cut) และยาแนว Joint sealant พื้น S1</t>
         </is>
       </c>
       <c r="D36" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: 46 ต้น (ตาม F2P 46 ฐาน) x 4.59 ม. (215.72/47 จาก S4.1) = 211.13 ม. x 44.1 กก./ม.</t>
+          <t>เพิ่ม: สมมติรอยต่อทุก 6 ม. ตามแนวกริด (9x54 + 8x60 ม.) รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="37" t="inlineStr">
         <is>
-          <t>2.5.2</t>
-        </is>
-      </c>
-      <c r="B37" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.5.1</t>
+        </is>
+      </c>
+      <c r="B37" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
-          <t>โครงถักหลังคา ช่วง 2 x 30 ม. 10 แนว (กริด A-J) สันหลังคา +14.10</t>
+          <t>เสาเหล็ก H250x175x44.1 กก./ม. บนหัวเสา คสล. +4.50 ถึง +9.00 พร้อมแผ่นเหล็กฐาน Anchor bolt</t>
         </is>
       </c>
       <c r="D37" s="37" t="inlineStr">
         <is>
-          <t>ประมาณการจากโมเดล (คอร์ด 2C-150x65x20x3.2, ค้ำ C-100x50x20x2.3) รอแบบ</t>
+          <t>แก้ไข: 46 ต้น (ตาม F2P 46 ฐาน) x 4.59 ม. (215.72/47 จาก S4.1) = 211.13 ม. x 44.1 กก./ม.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="37" t="inlineStr">
         <is>
-          <t>2.5.3</t>
+          <t>2.5.2</t>
         </is>
       </c>
       <c r="B38" s="40" t="inlineStr">
@@ -7694,19 +7698,19 @@
       </c>
       <c r="C38" s="37" t="inlineStr">
         <is>
-          <t>แปหลังคา C-125x50x20x3.2 และแปผนัง (Girt)</t>
+          <t>โครงถักหลังคา ช่วง 2 x 30 ม. 10 แนว (กริด A-J) สันหลังคา +14.10</t>
         </is>
       </c>
       <c r="D38" s="37" t="inlineStr">
         <is>
-          <t>ประมาณการจากโมเดล แปหลังคา ~2,730 ม. + แปผนัง 684 ม. รอแบบ</t>
+          <t>ประมาณการจากโมเดล (คอร์ด 2C-150x65x20x3.2, ค้ำ C-100x50x20x2.3) รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="37" t="inlineStr">
         <is>
-          <t>2.5.4</t>
+          <t>2.5.3</t>
         </is>
       </c>
       <c r="B39" s="40" t="inlineStr">
@@ -7716,37 +7720,41 @@
       </c>
       <c r="C39" s="37" t="inlineStr">
         <is>
-          <t>ค้ำยันหลังคา/ผนัง RB12 + Turnbuckle, Sag rod, แผ่นต่อ สลักเกลียว (จุดต่อ ~10%)</t>
+          <t>แปหลังคา C-125x50x20x3.2 และแปผนัง (Girt)</t>
         </is>
       </c>
       <c r="D39" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: ค้ำยัน 303 + จุดต่อ 10% ของ 2.5.1-2.5.3 (55,773) = 5,880 กก. ประมาณการ รอแบบ</t>
+          <t>ประมาณการจากโมเดล แปหลังคา ~2,730 ม. + แปผนัง 684 ม. รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="37" t="inlineStr">
         <is>
-          <t>2.5.5</t>
-        </is>
-      </c>
-      <c r="B40" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.5.4</t>
+        </is>
+      </c>
+      <c r="B40" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C40" s="37" t="inlineStr">
         <is>
-          <t>ทาสีกันสนิม 2 เที่ยว + สีทับหน้า 1 เที่ยว โครงสร้างเหล็กทั้งหมด</t>
-        </is>
-      </c>
-      <c r="D40" s="37" t="inlineStr"/>
+          <t>ค้ำยันหลังคา/ผนัง RB12 + Turnbuckle, Sag rod, แผ่นต่อ สลักเกลียว (จุดต่อ ~10%)</t>
+        </is>
+      </c>
+      <c r="D40" s="37" t="inlineStr">
+        <is>
+          <t>แก้ไข: ค้ำยัน 303 + จุดต่อ 10% ของ 2.5.1-2.5.3 (55,773) = 5,880 กก. ประมาณการ รอแบบ</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="37" t="inlineStr">
         <is>
-          <t>2.5.6</t>
+          <t>2.5.5</t>
         </is>
       </c>
       <c r="B41" s="39" t="inlineStr">
@@ -7756,19 +7764,15 @@
       </c>
       <c r="C41" s="37" t="inlineStr">
         <is>
-          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) ใต้แผ่นฐานเสาเหล็ก</t>
-        </is>
-      </c>
-      <c r="D41" s="37" t="inlineStr">
-        <is>
-          <t>เพิ่ม: เสาเหล็กบนหัวเสา คสล. C1 45 + C2 1 (S201)</t>
-        </is>
-      </c>
+          <t>ทาสีกันสนิม 2 เที่ยว + สีทับหน้า 1 เที่ยว โครงสร้างเหล็กทั้งหมด</t>
+        </is>
+      </c>
+      <c r="D41" s="37" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="37" t="inlineStr">
         <is>
-          <t>2.6.1</t>
+          <t>2.5.6</t>
         </is>
       </c>
       <c r="B42" s="39" t="inlineStr">
@@ -7778,63 +7782,63 @@
       </c>
       <c r="C42" s="37" t="inlineStr">
         <is>
-          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
+          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) ใต้แผ่นฐานเสาเหล็ก</t>
         </is>
       </c>
       <c r="D42" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: S4.1 36 ต้น ยาว 100.80 ม.</t>
+          <t>เพิ่ม: เสาเหล็กบนหัวเสา คสล. C1 45 + C2 1 (S201)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="37" t="inlineStr">
         <is>
-          <t>2.6.2</t>
-        </is>
-      </c>
-      <c r="B43" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.6.1</t>
+        </is>
+      </c>
+      <c r="B43" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
-          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
+          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
         </is>
       </c>
       <c r="D43" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ประมาณการ H200x100 ตารางคาน 3.00 ม.</t>
+          <t>เพิ่ม: S4.1 36 ต้น ยาว 100.80 ม.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="37" t="inlineStr">
         <is>
-          <t>2.6.3</t>
-        </is>
-      </c>
-      <c r="B44" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.6.2</t>
+        </is>
+      </c>
+      <c r="B44" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C44" s="37" t="inlineStr">
         <is>
-          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
+          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
         </is>
       </c>
       <c r="D44" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: S6.1 306.15 ตร.ม.</t>
+          <t>เพิ่ม: ประมาณการ H200x100 ตารางคาน 3.00 ม.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="37" t="inlineStr">
         <is>
-          <t>2.6.4</t>
+          <t>2.6.3</t>
         </is>
       </c>
       <c r="B45" s="39" t="inlineStr">
@@ -7844,19 +7848,19 @@
       </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
-          <t>บันไดเหล็กขึ้นชั้นลอย กว้าง ~1.40 ม. พร้อมราวกันตก</t>
+          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
         </is>
       </c>
       <c r="D45" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ตำแหน่ง DN แนวกริด D</t>
+          <t>เพิ่ม: S6.1 306.15 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="37" t="inlineStr">
         <is>
-          <t>2.6.5</t>
+          <t>2.6.4</t>
         </is>
       </c>
       <c r="B46" s="39" t="inlineStr">
@@ -7866,19 +7870,19 @@
       </c>
       <c r="C46" s="37" t="inlineStr">
         <is>
-          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
+          <t>บันไดเหล็กขึ้นชั้นลอย กว้าง ~1.40 ม. พร้อมราวกันตก</t>
         </is>
       </c>
       <c r="D46" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ขอบด้านเปิด 18 + 17 ม. หักช่องบันได 1.40 ม.</t>
+          <t>เพิ่ม: ตำแหน่ง DN แนวกริด D</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="37" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>2.6.5</t>
         </is>
       </c>
       <c r="B47" s="39" t="inlineStr">
@@ -7888,19 +7892,19 @@
       </c>
       <c r="C47" s="37" t="inlineStr">
         <is>
-          <t>หลังคาเมทัลชีทหนา 0.47 มม. พร้อมฉนวน PU 25 มม. (พื้นที่ตามลาด)</t>
+          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
         </is>
       </c>
       <c r="D47" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: จากโมเดล 2 ลาด 30.2 ม. x 55 ม. (สเปควัสดุรอยืนยัน)</t>
+          <t>เพิ่ม: ขอบด้านเปิด 18 + 17 ม. หักช่องบันได 1.40 ม.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="37" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="B48" s="39" t="inlineStr">
@@ -7910,19 +7914,19 @@
       </c>
       <c r="C48" s="37" t="inlineStr">
         <is>
-          <t>Jack roof กว้าง 6.00 ม. ยาว 42.00 ม. สัน +15.25 พร้อมตะแกรงระบายอากาศ</t>
+          <t>หลังคาเมทัลชีทหนา 0.47 มม. พร้อมฉนวน PU 25 มม. (พื้นที่ตามลาด)</t>
         </is>
       </c>
       <c r="D48" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A202</t>
+          <t>เพิ่ม: จากโมเดล 2 ลาด 30.2 ม. x 55 ม. (สเปควัสดุรอยืนยัน)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="37" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>3.1.2</t>
         </is>
       </c>
       <c r="B49" s="39" t="inlineStr">
@@ -7932,19 +7936,19 @@
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
-          <t>ครอบสัน ครอบข้าง แผ่นปิดเชิงชาย Flashing</t>
+          <t>Jack roof กว้าง 6.00 ม. ยาว 42.00 ม. สัน +15.25 พร้อมตะแกรงระบายอากาศ</t>
         </is>
       </c>
       <c r="D49" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม</t>
+          <t>เพิ่ม: A202</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>3.1.3</t>
         </is>
       </c>
       <c r="B50" s="39" t="inlineStr">
@@ -7954,107 +7958,107 @@
       </c>
       <c r="C50" s="37" t="inlineStr">
         <is>
-          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30 ม.</t>
+          <t>ครอบสัน ครอบข้าง แผ่นปิดเชิงชาย Flashing</t>
         </is>
       </c>
       <c r="D50" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ชายคาแนวกริด 1 และ 11</t>
+          <t>เพิ่ม</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="37" t="inlineStr">
         <is>
-          <t>3.1.5</t>
-        </is>
-      </c>
-      <c r="B51" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.1.4</t>
+        </is>
+      </c>
+      <c r="B51" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
-          <t>ท่อระบายน้ำฝน PVC Ø4" พร้อมอุปกรณ์ยึด</t>
+          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30 ม.</t>
         </is>
       </c>
       <c r="D51" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: 10 จุด x 10 ม. (สมมติ)</t>
+          <t>เพิ่ม: ชายคาแนวกริด 1 และ 11</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="37" t="inlineStr">
         <is>
-          <t>3.1.6</t>
-        </is>
-      </c>
-      <c r="B52" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.1.5</t>
+        </is>
+      </c>
+      <c r="B52" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C52" s="37" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท ระดับ +5.20 ถึงชายคา/จั่ว</t>
+          <t>ท่อระบายน้ำฝน PVC Ø4" พร้อมอุปกรณ์ยึด</t>
         </is>
       </c>
       <c r="D52" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: จากโมเดล ตาม A202</t>
+          <t>เพิ่ม: 10 จุด x 10 ม. (สมมติ)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
-          <t>3.1.7</t>
-        </is>
-      </c>
-      <c r="B53" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.1.6</t>
+        </is>
+      </c>
+      <c r="B53" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
-          <t>ตะแกรงกันนก/ช่องระบายอากาศ ระดับ +4.50 ถึง +5.20 รอบอาคาร</t>
+          <t>ผนังเมทัลชีท ระดับ +5.20 ถึงชายคา/จั่ว</t>
         </is>
       </c>
       <c r="D53" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ช่องระหว่างผนังก่อกับเมทัลชีท (A202) หักประตูม้วน 12 ม.</t>
+          <t>เพิ่ม: จากโมเดล ตาม A202</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="37" t="inlineStr">
         <is>
-          <t>3.2.1</t>
-        </is>
-      </c>
-      <c r="B54" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>3.1.7</t>
+        </is>
+      </c>
+      <c r="B54" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C54" s="37" t="inlineStr">
         <is>
-          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ม. +0.50 ถึง +4.35 (ต่ำกว่าหัวเสา คสล. 0.15 ม.)</t>
+          <t>ตะแกรงกันนก/ช่องระบายอากาศ ระดับ +4.50 ถึง +5.20 รอบอาคาร</t>
         </is>
       </c>
       <c r="D54" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: ผนัง 36 ช่วง ยาวสุทธิ 205.20 ม. x 3.85 ม. หักประตู D1 2 ช่อง, เสาเอ็น, คานเอ็น (ดูชีต 'ผนัง-รายละเอียด')</t>
+          <t>เพิ่ม: ช่องระหว่างผนังก่อกับเมทัลชีท (A202) หักประตูม้วน 12 ม.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="37" t="inlineStr">
         <is>
-          <t>3.2.2</t>
+          <t>3.2.1</t>
         </is>
       </c>
       <c r="B55" s="38" t="inlineStr">
@@ -8064,41 +8068,41 @@
       </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
-          <t>ฉาบปูนผนังก่อ คานเอ็น คานทับหลัง และเสาเอ็น 2 ด้าน (+0.50 ถึง +4.50)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ม. +0.50 ถึง +4.35 (ต่ำกว่าหัวเสา คสล. 0.15 ม.)</t>
         </is>
       </c>
       <c r="D55" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: 205.20 ม. x 4.00 ม. x 2 ด้าน หักประตู D1</t>
+          <t>แก้ไข: ผนัง 36 ช่วง ยาวสุทธิ 205.20 ม. x 3.85 ม. หักประตู D1 2 ช่อง, เสาเอ็น, คานเอ็น (ดูชีต 'ผนัง-รายละเอียด')</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="37" t="inlineStr">
         <is>
-          <t>3.2.3</t>
-        </is>
-      </c>
-      <c r="B56" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.2.2</t>
+        </is>
+      </c>
+      <c r="B56" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C56" s="37" t="inlineStr">
         <is>
-          <t>คานทับหลัง คสล. 0.15x0.15 ม. ระดับ +4.35 ถึง +4.50 (คอนกรีต ไม้แบบ)</t>
+          <t>ฉาบปูนผนังก่อ คานเอ็น คานทับหลัง และเสาเอ็น 2 ด้าน (+0.50 ถึง +4.50)</t>
         </is>
       </c>
       <c r="D56" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ผู้ว่าจ้างกำหนด คอนกรีต 4.62 ลบ.ม. ไม้แบบ 61.56 ตร.ม.</t>
+          <t>แก้ไข: 205.20 ม. x 4.00 ม. x 2 ด้าน หักประตู D1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="37" t="inlineStr">
         <is>
-          <t>3.2.4</t>
+          <t>3.2.3</t>
         </is>
       </c>
       <c r="B57" s="39" t="inlineStr">
@@ -8108,19 +8112,19 @@
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
-          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังวงกบประตู +2.60 (คอนกรีต ไม้แบบ)</t>
+          <t>คานทับหลัง คสล. 0.15x0.15 ม. ระดับ +4.35 ถึง +4.50 (คอนกรีต ไม้แบบ)</t>
         </is>
       </c>
       <c r="D57" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ผนังสูง 3.85 ม. &gt; 3 ม. ต้องมีคานเอ็นกลางผนัง คอนกรีต 3.08 ลบ.ม. ไม้แบบ 41.04 ตร.ม.</t>
+          <t>เพิ่ม: ผู้ว่าจ้างกำหนด คอนกรีต 4.62 ลบ.ม. ไม้แบบ 61.56 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="37" t="inlineStr">
         <is>
-          <t>3.2.5</t>
+          <t>3.2.4</t>
         </is>
       </c>
       <c r="B58" s="39" t="inlineStr">
@@ -8130,63 +8134,63 @@
       </c>
       <c r="C58" s="37" t="inlineStr">
         <is>
-          <t>เสาเอ็น คสล. 0.15x0.10 ม. สูง 3.85 ม. (กลางช่วงเสา 6 ม. และข้างวงกบประตู)</t>
+          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังวงกบประตู +2.60 (คอนกรีต ไม้แบบ)</t>
         </is>
       </c>
       <c r="D58" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ยาวรวม 146.30 ม. คอนกรีต 2.19 ลบ.ม. ไม้แบบ 29.26 ตร.ม.</t>
+          <t>เพิ่ม: ผนังสูง 3.85 ม. &gt; 3 ม. ต้องมีคานเอ็นกลางผนัง คอนกรีต 3.08 ลบ.ม. ไม้แบบ 41.04 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="37" t="inlineStr">
         <is>
-          <t>3.2.6</t>
-        </is>
-      </c>
-      <c r="B59" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.2.5</t>
+        </is>
+      </c>
+      <c r="B59" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริมคานทับหลัง คานเอ็น เสาเอ็น</t>
+          <t>เสาเอ็น คสล. 0.15x0.10 ม. สูง 3.85 ม. (กลางช่วงเสา 6 ม. และข้างวงกบประตู)</t>
         </is>
       </c>
       <c r="D59" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม</t>
+          <t>เพิ่ม: ยาวรวม 146.30 ม. คอนกรีต 2.19 ลบ.ม. ไม้แบบ 29.26 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="37" t="inlineStr">
         <is>
-          <t>3.2.7</t>
-        </is>
-      </c>
-      <c r="B60" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="B60" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C60" s="37" t="inlineStr">
         <is>
-          <t>ฉาบปูนเสา คสล. C1/C2 ที่ผิวเปิด (+0.50 ถึง +4.50)</t>
+          <t>เหล็กเสริมคานทับหลัง คานเอ็น เสาเอ็น</t>
         </is>
       </c>
       <c r="D60" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: เสาแนวผนัง 38 ต้น x 1.30 ม. + เสากลางอาคาร 8 ต้น x 1.60 ม. x สูง 4.00 ม.</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="37" t="inlineStr">
         <is>
-          <t>3.2.8</t>
+          <t>3.2.7</t>
         </is>
       </c>
       <c r="B61" s="39" t="inlineStr">
@@ -8196,63 +8200,63 @@
       </c>
       <c r="C61" s="37" t="inlineStr">
         <is>
-          <t>จับเซี้ยมมุมเสา คสล. มุมผนัง ขอบคานทับหลัง และขอบช่องประตู ก่อนฉาบเสาและผนัง</t>
+          <t>ฉาบปูนเสา คสล. C1/C2 ที่ผิวเปิด (+0.50 ถึง +4.50)</t>
         </is>
       </c>
       <c r="D61" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: มุมเสาแนวผนัง 608.0 + มุมเสากลางอาคาร 128.0 + ขอบบนคานทับหลัง 2 ด้าน 410.4 + ขอบช่องประตู D1 20.8 ม.</t>
+          <t>เพิ่ม: เสาแนวผนัง 38 ต้น x 1.30 ม. + เสากลางอาคาร 8 ต้น x 1.60 ม. x สูง 4.00 ม.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="37" t="inlineStr">
         <is>
-          <t>3.3.1</t>
-        </is>
-      </c>
-      <c r="B62" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>3.2.8</t>
+        </is>
+      </c>
+      <c r="B62" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C62" s="37" t="inlineStr">
         <is>
-          <t>พื้นขัดมันผสม Floor Hardener</t>
+          <t>จับเซี้ยมมุมเสา คสล. มุมผนัง ขอบคานทับหลัง และขอบช่องประตู ก่อนฉาบเสาและผนัง</t>
         </is>
       </c>
       <c r="D62" s="37" t="inlineStr">
         <is>
-          <t>เดิม 3,240 → พื้นที่ S1 (S6.1)</t>
+          <t>เพิ่ม: มุมเสาแนวผนัง 608.0 + มุมเสากลางอาคาร 128.0 + ขอบบนคานทับหลัง 2 ด้าน 410.4 + ขอบช่องประตู D1 20.8 ม.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="37" t="inlineStr">
         <is>
-          <t>3.4.1</t>
-        </is>
-      </c>
-      <c r="B63" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.3.1</t>
+        </is>
+      </c>
+      <c r="B63" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
-          <t>ประตูม้วนเหล็กไฟฟ้า ~6.00x4.00 ม. ทางลาดขนส่ง</t>
+          <t>พื้นขัดมันผสม Floor Hardener</t>
         </is>
       </c>
       <c r="D63" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ตำแหน่งตาม A101 ขนาดรอยืนยัน</t>
+          <t>เดิม 3,240 → พื้นที่ S1 (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="37" t="inlineStr">
         <is>
-          <t>3.4.2</t>
+          <t>3.4.1</t>
         </is>
       </c>
       <c r="B64" s="40" t="inlineStr">
@@ -8262,41 +8266,41 @@
       </c>
       <c r="C64" s="37" t="inlineStr">
         <is>
-          <t>ประตู D1/D2/D4 และหน้าต่าง ตามแบบ A101</t>
+          <t>ประตูม้วนเหล็กไฟฟ้า ~6.00x4.00 ม. ทางลาดขนส่ง</t>
         </is>
       </c>
       <c r="D64" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: รอตารางประตู-หน้าต่าง</t>
+          <t>เพิ่ม: ตำแหน่งตาม A101 ขนาดรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="37" t="inlineStr">
         <is>
-          <t>3.5.1</t>
-        </is>
-      </c>
-      <c r="B65" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.4.2</t>
+        </is>
+      </c>
+      <c r="B65" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C65" s="37" t="inlineStr">
         <is>
-          <t>ทาสีผนังและเสา ภายใน-ภายนอก (รองพื้น + ทับหน้า 2 เที่ยว)</t>
+          <t>ประตู D1/D2/D4 และหน้าต่าง ตามแบบ A101</t>
         </is>
       </c>
       <c r="D65" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: เท่ากับพื้นที่ฉาบ 3.2.2 + 3.2.7</t>
+          <t>เพิ่ม: รอตารางประตู-หน้าต่าง</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t>3.6.1</t>
+          <t>3.5.1</t>
         </is>
       </c>
       <c r="B66" s="39" t="inlineStr">
@@ -8306,19 +8310,19 @@
       </c>
       <c r="C66" s="37" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. (ผนัง ประตูกันไฟ พื้น ฝ้า)</t>
+          <t>ทาสีผนังและเสา ภายใน-ภายนอก (รองพื้น + ทับหน้า 2 เที่ยว)</t>
         </is>
       </c>
       <c r="D66" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A101</t>
+          <t>แก้ไข: เท่ากับพื้นที่ฉาบ 3.2.2 + 3.2.7</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="37" t="inlineStr">
         <is>
-          <t>3.6.2</t>
+          <t>3.6.1</t>
         </is>
       </c>
       <c r="B67" s="39" t="inlineStr">
@@ -8328,7 +8332,7 @@
       </c>
       <c r="C67" s="37" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. พร้อมขอบกั้นรั่วไหล</t>
+          <t>ห้อง MDB 17.79 ตร.ม. (ผนัง ประตูกันไฟ พื้น ฝ้า)</t>
         </is>
       </c>
       <c r="D67" s="37" t="inlineStr">
@@ -8340,29 +8344,29 @@
     <row r="68">
       <c r="A68" s="37" t="inlineStr">
         <is>
-          <t>3.6.3</t>
-        </is>
-      </c>
-      <c r="B68" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.6.2</t>
+        </is>
+      </c>
+      <c r="B68" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C68" s="37" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ 2.40 x 8.00 ม. (สุขภัณฑ์ กระเบื้อง ระบบสุขาภิบาลภายใน)</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. พร้อมขอบกั้นรั่วไหล</t>
         </is>
       </c>
       <c r="D68" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A101/S201 รอแบบสถาปัตย์</t>
+          <t>เพิ่ม: A101</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="37" t="inlineStr">
         <is>
-          <t>3.6.4</t>
+          <t>3.6.3</t>
         </is>
       </c>
       <c r="B69" s="40" t="inlineStr">
@@ -8372,41 +8376,41 @@
       </c>
       <c r="C69" s="37" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (กริด 8-10)</t>
+          <t>อาคารห้องน้ำ 2.40 x 8.00 ม. (สุขภัณฑ์ กระเบื้อง ระบบสุขาภิบาลภายใน)</t>
         </is>
       </c>
       <c r="D69" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: เห็นในผัง A101 รอแบบ</t>
+          <t>เพิ่ม: A101/S201 รอแบบสถาปัตย์</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="37" t="inlineStr">
         <is>
-          <t>3.6.5</t>
-        </is>
-      </c>
-      <c r="B70" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.6.4</t>
+        </is>
+      </c>
+      <c r="B70" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C70" s="37" t="inlineStr">
         <is>
-          <t>บันได/ชานพัก คสล. หน้าประตู D1 ภายนอก (พื้น +0.50 ถนน ±0.00)</t>
+          <t>ห้องประกอบแนวกริด A (กริด 8-10)</t>
         </is>
       </c>
       <c r="D70" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ประตู D1 ผนังแนวกริด 1 และ 11 (A101) ระดับต่างกัน 0.50 ม.</t>
+          <t>เพิ่ม: เห็นในผัง A101 รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="37" t="inlineStr">
         <is>
-          <t>4.1.1</t>
+          <t>3.6.5</t>
         </is>
       </c>
       <c r="B71" s="39" t="inlineStr">
@@ -8416,19 +8420,19 @@
       </c>
       <c r="C71" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับพื้นถนนรอบอาคาร (I22-22) รวมค่าตอก</t>
+          <t>บันได/ชานพัก คสล. หน้าประตู D1 ภายนอก (พื้น +0.50 ถนน ±0.00)</t>
         </is>
       </c>
       <c r="D71" s="37" t="inlineStr">
         <is>
-          <t>ตาราง S2 = 249; นับจากผัง S201 ได้ 232 (ยืนยันจำนวน)</t>
+          <t>เพิ่ม: ประตู D1 ผนังแนวกริด 1 และ 11 (A101) ระดับต่างกัน 0.50 ม.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="37" t="inlineStr">
         <is>
-          <t>4.1.2</t>
+          <t>4.1.1</t>
         </is>
       </c>
       <c r="B72" s="39" t="inlineStr">
@@ -8438,19 +8442,19 @@
       </c>
       <c r="C72" s="37" t="inlineStr">
         <is>
-          <t>ฐาน F1A 0.60x0.60x0.30 ม. รับพื้นถนน</t>
+          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับพื้นถนนรอบอาคาร (I22-22) รวมค่าตอก</t>
         </is>
       </c>
       <c r="D72" s="37" t="inlineStr">
         <is>
-          <t>คอนกรีต 26.78, ทราย 35.86, คอนกรีตหยาบ 6.10 ลบ.ม. (S1.1)</t>
+          <t>กลุ่มเข็มถนน: ผู้ว่าจ้างยืนยัน 249 ต้น (ผัง S201/S202 แสดงตำแหน่ง 232 ต้น ขอตำแหน่งอีก 17 ต้นจากผู้ออกแบบ)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="37" t="inlineStr">
         <is>
-          <t>4.1.3</t>
+          <t>4.1.2</t>
         </is>
       </c>
       <c r="B73" s="39" t="inlineStr">
@@ -8460,19 +8464,19 @@
       </c>
       <c r="C73" s="37" t="inlineStr">
         <is>
-          <t>พื้นถนน S2 คสล. หนา 0.15 ม. TOP ±0.00 พร้อมรอยต่อ/ตัดรอยต่อ</t>
+          <t>ฐาน F1A 0.60x0.60x0.30 ม. รับพื้นถนน</t>
         </is>
       </c>
       <c r="D73" s="37" t="inlineStr">
         <is>
-          <t>คอนกรีต 366.10 ลบ.ม. (S6.1)</t>
+          <t>ตามเข็มถนน 249 ต้น คอนกรีต 26.78, ทราย 35.86, คอนกรีตหยาบ 6.10 ลบ.ม. (S1.1)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="37" t="inlineStr">
         <is>
-          <t>4.1.4</t>
+          <t>4.1.3</t>
         </is>
       </c>
       <c r="B74" s="39" t="inlineStr">
@@ -8482,41 +8486,41 @@
       </c>
       <c r="C74" s="37" t="inlineStr">
         <is>
-          <t>พื้น AF01 / SF02 ระดับถนน</t>
+          <t>พื้นถนน S2 คสล. หนา 0.15 ม. TOP ±0.00 พร้อมรอยต่อ/ตัดรอยต่อ</t>
         </is>
       </c>
       <c r="D74" s="37" t="inlineStr">
         <is>
-          <t>AF01 16.88 + SF02 93.26 ตร.ม. คอนกรีต 25.76 ลบ.ม. (S6.1)</t>
+          <t>คอนกรีต 366.10 ลบ.ม. (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="37" t="inlineStr">
         <is>
-          <t>4.1.5</t>
-        </is>
-      </c>
-      <c r="B75" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.1.4</t>
+        </is>
+      </c>
+      <c r="B75" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C75" s="37" t="inlineStr">
         <is>
-          <t>ทราย/หินคลุกรองใต้พื้นถนน S2 หนา 0.10 ม. บดอัด</t>
+          <t>พื้น AF01 / SF02 ระดับถนน</t>
         </is>
       </c>
       <c r="D75" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: 2,440.69 ตร.ม. x 0.10 ม. (ความหนาสมมติ รอแบบ)</t>
+          <t>AF01 16.88 + SF02 93.26 ตร.ม. คอนกรีต 25.76 ลบ.ม. (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="37" t="inlineStr">
         <is>
-          <t>4.1.6</t>
+          <t>4.1.5</t>
         </is>
       </c>
       <c r="B76" s="40" t="inlineStr">
@@ -8526,41 +8530,41 @@
       </c>
       <c r="C76" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม/ตะแกรงเหล็ก พื้นถนน และฐาน F1A</t>
+          <t>ทราย/หินคลุกรองใต้พื้นถนน S2 หนา 0.10 ม. บดอัด</t>
         </is>
       </c>
       <c r="D76" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม</t>
+          <t>เพิ่ม: 2,440.69 ตร.ม. x 0.10 ม. (ความหนาสมมติ รอแบบ)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="37" t="inlineStr">
         <is>
-          <t>4.2.1</t>
-        </is>
-      </c>
-      <c r="B77" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>4.1.6</t>
+        </is>
+      </c>
+      <c r="B77" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C77" s="37" t="inlineStr">
         <is>
-          <t>ทางลาดขนส่ง คสล. กว้าง 6.00 ม. (ด้านเหนือแนวกริด 5-6 และด้านใต้แนวกริด 7-8)</t>
+          <t>เหล็กเสริม/ตะแกรงเหล็ก พื้นถนน และฐาน F1A</t>
         </is>
       </c>
       <c r="D77" s="37" t="inlineStr">
         <is>
-          <t>A101/S202 ขนาดวัดจากผัง</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="37" t="inlineStr">
         <is>
-          <t>4.3.1</t>
+          <t>4.2.1</t>
         </is>
       </c>
       <c r="B78" s="39" t="inlineStr">
@@ -8570,59 +8574,59 @@
       </c>
       <c r="C78" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
+          <t>ทางลาดขนส่ง คสล. กว้าง 6.00 ม. (ด้านเหนือแนวกริด 5-6 และด้านใต้แนวกริด 7-8)</t>
         </is>
       </c>
       <c r="D78" s="37" t="inlineStr">
         <is>
-          <t>S2 / S201</t>
+          <t>A101/S202 ขนาดวัดจากผัง</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="37" t="inlineStr">
         <is>
-          <t>4.3.2</t>
-        </is>
-      </c>
-      <c r="B79" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.3.1</t>
+        </is>
+      </c>
+      <c r="B79" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C79" s="37" t="inlineStr">
         <is>
-          <t>ฐานหม้อแปลง คสล. (ขนาดรอแบบขยาย)</t>
-        </is>
-      </c>
-      <c r="D79" s="37" t="inlineStr"/>
+          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
+        </is>
+      </c>
+      <c r="D79" s="37" t="inlineStr">
+        <is>
+          <t>S2 / S201</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="37" t="inlineStr">
         <is>
-          <t>4.4.1</t>
-        </is>
-      </c>
-      <c r="B80" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>4.3.2</t>
+        </is>
+      </c>
+      <c r="B80" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C80" s="37" t="inlineStr">
         <is>
-          <t>ขุดดินถังเก็บน้ำใต้ดิน ~12.12 x 6.63 ม. ลึก 3.00 ม. และขนทิ้ง</t>
-        </is>
-      </c>
-      <c r="D80" s="37" t="inlineStr">
-        <is>
-          <t>เพิ่ม: ขนาดจากเวกเตอร์ S201/S202 ลึกจาก ±0.00 ถึงใต้คอนกรีตหยาบ -3.00</t>
-        </is>
-      </c>
+          <t>ฐานหม้อแปลง คสล. (ขนาดรอแบบขยาย)</t>
+        </is>
+      </c>
+      <c r="D80" s="37" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="37" t="inlineStr">
         <is>
-          <t>4.4.2</t>
+          <t>4.4.1</t>
         </is>
       </c>
       <c r="B81" s="39" t="inlineStr">
@@ -8632,41 +8636,41 @@
       </c>
       <c r="C81" s="37" t="inlineStr">
         <is>
-          <t>พื้นถังเก็บน้ำใต้ดิน คสล. หนา 0.25 ม. (TF -2.60 / BF -2.85) พร้อมคอนกรีตหยาบ/ทราย</t>
+          <t>ขุดดินถังเก็บน้ำใต้ดิน ~12.12 x 6.63 ม. ลึก 3.00 ม. และขนทิ้ง</t>
         </is>
       </c>
       <c r="D81" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: 12.12 x 6.63 ม. คอนกรีต 20.09 ลบ.ม. (S202)</t>
+          <t>เพิ่ม: ขนาดจากเวกเตอร์ S201/S202 ลึกจาก ±0.00 ถึงใต้คอนกรีตหยาบ -3.00</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="37" t="inlineStr">
         <is>
-          <t>4.4.3</t>
-        </is>
-      </c>
-      <c r="B82" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.4.2</t>
+        </is>
+      </c>
+      <c r="B82" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C82" s="37" t="inlineStr">
         <is>
-          <t>ผนัง ฝา ช่องเปิด บ่อพัก บันไดลิง และกันซึม ถังเก็บน้ำใต้ดิน</t>
+          <t>พื้นถังเก็บน้ำใต้ดิน คสล. หนา 0.25 ม. (TF -2.60 / BF -2.85) พร้อมคอนกรีตหยาบ/ทราย</t>
         </is>
       </c>
       <c r="D82" s="37" t="inlineStr">
         <is>
-          <t>รอแบบขยาย (S202 แสดงเฉพาะพื้นถัง)</t>
+          <t>เพิ่ม: 12.12 x 6.63 ม. คอนกรีต 20.09 ลบ.ม. (S202)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="37" t="inlineStr">
         <is>
-          <t>4.4.4</t>
+          <t>4.4.3</t>
         </is>
       </c>
       <c r="B83" s="40" t="inlineStr">
@@ -8676,19 +8680,19 @@
       </c>
       <c r="C83" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริมถังเก็บน้ำใต้ดิน</t>
+          <t>ผนัง ฝา ช่องเปิด บ่อพัก บันไดลิง และกันซึม ถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="D83" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม</t>
+          <t>รอแบบขยาย (S202 แสดงเฉพาะพื้นถัง)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="37" t="inlineStr">
         <is>
-          <t>4.5.1</t>
+          <t>4.4.4</t>
         </is>
       </c>
       <c r="B84" s="40" t="inlineStr">
@@ -8698,19 +8702,19 @@
       </c>
       <c r="C84" s="37" t="inlineStr">
         <is>
-          <t>รางระบายน้ำ คสล. พร้อมฝาปิด ตามแนวเขตที่ดิน</t>
+          <t>เหล็กเสริมถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="D84" s="37" t="inlineStr">
         <is>
-          <t>A101 ขนาดรางรอแบบขยาย</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="37" t="inlineStr">
         <is>
-          <t>4.5.2</t>
+          <t>4.5.1</t>
         </is>
       </c>
       <c r="B85" s="40" t="inlineStr">
@@ -8720,63 +8724,63 @@
       </c>
       <c r="C85" s="37" t="inlineStr">
         <is>
-          <t>บ่อพัก/บ่อบำบัด และจุดเชื่อมท่อระบายสาธารณะ</t>
+          <t>รางระบายน้ำ คสล. พร้อมฝาปิด ตามแนวเขตที่ดิน</t>
         </is>
       </c>
       <c r="D85" s="37" t="inlineStr">
         <is>
-          <t>รอแบบ</t>
+          <t>A101 ขนาดรางรอแบบขยาย</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="37" t="inlineStr">
         <is>
-          <t>4.5.3</t>
-        </is>
-      </c>
-      <c r="B86" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>4.5.2</t>
+        </is>
+      </c>
+      <c r="B86" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C86" s="37" t="inlineStr">
         <is>
-          <t>ท่อระบายน้ำฝนใต้ดิน PVC Ø4" จากท่อลงถึงรางระบายน้ำ</t>
+          <t>บ่อพัก/บ่อบำบัด และจุดเชื่อมท่อระบายสาธารณะ</t>
         </is>
       </c>
       <c r="D86" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ท่อลง 10 จุด (3.1.5)</t>
+          <t>รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="37" t="inlineStr">
         <is>
-          <t>4.6.1</t>
-        </is>
-      </c>
-      <c r="B87" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.5.3</t>
+        </is>
+      </c>
+      <c r="B87" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C87" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-260x260 + ฐาน 0.66x0.66 ม. แนวเขตที่ดินด้านใต้และตะวันออก (ไม่มีใน BOQ/ตาราง S2)</t>
+          <t>ท่อระบายน้ำฝนใต้ดิน PVC Ø4" จากท่อลงถึงรางระบายน้ำ</t>
         </is>
       </c>
       <c r="D87" s="37" t="inlineStr">
         <is>
-          <t>พบในผัง S201 16 จุด ยังไม่ทราบหน้าที่ (เสารั้ว/เสาไฟ/ป้าย?) สอบถามผู้ออกแบบ</t>
+          <t>เพิ่ม: ท่อลง 10 จุด (3.1.5)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="37" t="inlineStr">
         <is>
-          <t>4.6.2</t>
+          <t>4.6.1</t>
         </is>
       </c>
       <c r="B88" s="40" t="inlineStr">
@@ -8786,19 +8790,19 @@
       </c>
       <c r="C88" s="37" t="inlineStr">
         <is>
-          <t>รั้วถาวร / ประตูทางเข้าโครงการ</t>
+          <t>เสาเข็ม I-260x260 + ฐาน 0.66x0.66 ม. แนวเขตที่ดินด้านใต้และตะวันออก (ไม่มีใน BOQ/ตาราง S2)</t>
         </is>
       </c>
       <c r="D88" s="37" t="inlineStr">
         <is>
-          <t>ไม่มีในแบบ ยืนยันว่าอยู่ในขอบเขตหรือไม่</t>
+          <t>พบในผัง S201 16 จุด ยังไม่ทราบหน้าที่ (เสารั้ว/เสาไฟ/ป้าย?) สอบถามผู้ออกแบบ</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="37" t="inlineStr">
         <is>
-          <t>5.1.1</t>
+          <t>4.6.2</t>
         </is>
       </c>
       <c r="B89" s="40" t="inlineStr">
@@ -8808,19 +8812,19 @@
       </c>
       <c r="C89" s="37" t="inlineStr">
         <is>
-          <t>ระบบไฟฟ้าแสงสว่างและเต้ารับภายในอาคารโกดัง 3,240 ตร.ม. และไฟส่องสว่างภายนอก</t>
+          <t>รั้วถาวร / ประตูทางเข้าโครงการ</t>
         </is>
       </c>
       <c r="D89" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum</t>
+          <t>ไม่มีในแบบ ยืนยันว่าอยู่ในขอบเขตหรือไม่</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="37" t="inlineStr">
         <is>
-          <t>5.1.2</t>
+          <t>5.1.1</t>
         </is>
       </c>
       <c r="B90" s="40" t="inlineStr">
@@ -8830,19 +8834,19 @@
       </c>
       <c r="C90" s="37" t="inlineStr">
         <is>
-          <t>สายเมนและท่อร้อยสายใต้ดินจากหม้อแปลงถึงห้อง MDB</t>
+          <t>ระบบไฟฟ้าแสงสว่างและเต้ารับภายในอาคารโกดัง 3,240 ตร.ม. และไฟส่องสว่างภายนอก</t>
         </is>
       </c>
       <c r="D90" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum (ระยะประมาณ 10 ม.)</t>
+          <t>เพิ่ม: Provisional sum</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="37" t="inlineStr">
         <is>
-          <t>5.1.3</t>
+          <t>5.1.2</t>
         </is>
       </c>
       <c r="B91" s="40" t="inlineStr">
@@ -8852,19 +8856,19 @@
       </c>
       <c r="C91" s="37" t="inlineStr">
         <is>
-          <t>ระบบป้องกันฟ้าผ่าและสายดิน อาคารสูง +15.25 ม.</t>
+          <t>สายเมนและท่อร้อยสายใต้ดินจากหม้อแปลงถึงห้อง MDB</t>
         </is>
       </c>
       <c r="D91" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum</t>
+          <t>เพิ่ม: Provisional sum (ระยะประมาณ 10 ม.)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="37" t="inlineStr">
         <is>
-          <t>5.1.4</t>
+          <t>5.1.3</t>
         </is>
       </c>
       <c r="B92" s="40" t="inlineStr">
@@ -8874,7 +8878,7 @@
       </c>
       <c r="C92" s="37" t="inlineStr">
         <is>
-          <t>ระบบสุขาภิบาลและถังบำบัดน้ำเสียสำเร็จรูป อาคารห้องน้ำ</t>
+          <t>ระบบป้องกันฟ้าผ่าและสายดิน อาคารสูง +15.25 ม.</t>
         </is>
       </c>
       <c r="D92" s="37" t="inlineStr">
@@ -8886,7 +8890,7 @@
     <row r="93">
       <c r="A93" s="37" t="inlineStr">
         <is>
-          <t>5.1.5</t>
+          <t>5.1.4</t>
         </is>
       </c>
       <c r="B93" s="40" t="inlineStr">
@@ -8896,7 +8900,7 @@
       </c>
       <c r="C93" s="37" t="inlineStr">
         <is>
-          <t>ระบบน้ำประปา ปั๊มน้ำ และท่อจากถังเก็บน้ำใต้ดิน</t>
+          <t>ระบบสุขาภิบาลและถังบำบัดน้ำเสียสำเร็จรูป อาคารห้องน้ำ</t>
         </is>
       </c>
       <c r="D93" s="37" t="inlineStr">
@@ -8908,65 +8912,73 @@
     <row r="94">
       <c r="A94" s="37" t="inlineStr">
         <is>
+          <t>5.1.5</t>
+        </is>
+      </c>
+      <c r="B94" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
+        </is>
+      </c>
+      <c r="C94" s="37" t="inlineStr">
+        <is>
+          <t>ระบบน้ำประปา ปั๊มน้ำ และท่อจากถังเก็บน้ำใต้ดิน</t>
+        </is>
+      </c>
+      <c r="D94" s="37" t="inlineStr">
+        <is>
+          <t>เพิ่ม: Provisional sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="37" t="inlineStr">
+        <is>
           <t>5.1.6</t>
         </is>
       </c>
-      <c r="B94" s="40" t="inlineStr">
+      <c r="B95" s="40" t="inlineStr">
         <is>
           <t>รอข้อมูล</t>
         </is>
       </c>
-      <c r="C94" s="37" t="inlineStr">
+      <c r="C95" s="37" t="inlineStr">
         <is>
           <t>อุปกรณ์ดับเพลิง ป้ายทางออก ไฟฉุกเฉิน และระบบแจ้งเหตุเพลิงไหม้</t>
         </is>
       </c>
-      <c r="D94" s="37" t="inlineStr">
+      <c r="D95" s="37" t="inlineStr">
         <is>
           <t>เพิ่ม: Provisional sum</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="37" t="n"/>
-      <c r="B95" s="37" t="n"/>
-      <c r="C95" s="37" t="n"/>
-      <c r="D95" s="37" t="n"/>
-    </row>
     <row r="96">
-      <c r="A96" s="37" t="inlineStr"/>
-      <c r="B96" s="41" t="inlineStr">
-        <is>
-          <t>ข้อสังเกต</t>
-        </is>
-      </c>
-      <c r="C96" s="37" t="inlineStr"/>
-      <c r="D96" s="37" t="inlineStr"/>
+      <c r="A96" s="37" t="n"/>
+      <c r="B96" s="37" t="n"/>
+      <c r="C96" s="37" t="n"/>
+      <c r="D96" s="37" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="37" t="inlineStr"/>
-      <c r="B97" s="37" t="inlineStr">
-        <is>
-          <t>ขอบเขต</t>
-        </is>
-      </c>
-      <c r="C97" s="37" t="inlineStr">
-        <is>
-          <t>งานระบบไฟฟ้า ประปา สุขาภิบาล ดับเพลิง (MEP) ไม่มีแบบ เสนอเป็นเงินสำรองในหมวด 5 ให้ผู้ว่าจ้างยืนยันขอบเขตก่อนสรุปราคา</t>
-        </is>
-      </c>
+      <c r="B97" s="41" t="inlineStr">
+        <is>
+          <t>ข้อสังเกต</t>
+        </is>
+      </c>
+      <c r="C97" s="37" t="inlineStr"/>
       <c r="D97" s="37" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="37" t="inlineStr"/>
       <c r="B98" s="37" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>ขอบเขต</t>
         </is>
       </c>
       <c r="C98" s="37" t="inlineStr">
         <is>
-          <t>กรอบชื่อแบบทุกแผ่นระบุ 'แบบก่อสร้างบ้านพักอาศัย คสล 1 ชั้น' และ Date 03/31/22 ควรแก้ก่อนแนบประกอบใบเสนอราคา</t>
+          <t>งานระบบไฟฟ้า ประปา สุขาภิบาล ดับเพลิง (MEP) ไม่มีแบบ เสนอเป็นเงินสำรองในหมวด 5 ให้ผู้ว่าจ้างยืนยันขอบเขตก่อนสรุปราคา</t>
         </is>
       </c>
       <c r="D98" s="37" t="inlineStr"/>
@@ -8980,7 +8992,7 @@
       </c>
       <c r="C99" s="37" t="inlineStr">
         <is>
-          <t>แบบไม่มีลูกศรทิศเหนือ (North arrow) ต้องระบุเพื่อวางทิศอาคารบนที่ดินจริง</t>
+          <t>กรอบชื่อแบบทุกแผ่นระบุ 'แบบก่อสร้างบ้านพักอาศัย คสล 1 ชั้น' และ Date 03/31/22 ควรแก้ก่อนแนบประกอบใบเสนอราคา</t>
         </is>
       </c>
       <c r="D99" s="37" t="inlineStr"/>
@@ -8994,7 +9006,7 @@
       </c>
       <c r="C100" s="37" t="inlineStr">
         <is>
-          <t>ตาราง S2 นับเข็ม 737 ต้น แต่ผัง S201 นับได้ 734 ต้น (+16 ต้นใต้ฐาน 0.66 ม. ที่ไม่อยู่ในตาราง) และ F2P ผู้ว่าจ้างยืนยัน 46 ฐาน (ตาราง S1.1 นับ 47 ผิด เสาเหล็ก H250x175 จึงเป็น 46 ต้น)</t>
+          <t>แบบไม่มีลูกศรทิศเหนือ ผู้ว่าจ้างยืนยันให้ด้านแนวกริด A เป็นทิศเหนือสำหรับทำแบบ</t>
         </is>
       </c>
       <c r="D100" s="37" t="inlineStr"/>
@@ -9003,12 +9015,12 @@
       <c r="A101" s="37" t="inlineStr"/>
       <c r="B101" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม</t>
+          <t>แบบ</t>
         </is>
       </c>
       <c r="C101" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม คสล. ทุกรายการรอเอกสารการออกแบบเหล็กเสริมจากผู้ออกแบบ ตัวเลขในหมายเหตุเป็นค่าอ้างอิงเท่านั้น ไม่ใช้เป็นปริมาณ</t>
+          <t>ตาราง S2 นับเข็ม 737 ต้น แต่ผัง S201 นับได้ 734 ต้น (+16 ต้นใต้ฐาน 0.66 ม. ที่ไม่อยู่ในตาราง) และ F2P ผู้ว่าจ้างยืนยัน 46 ฐาน (ตาราง S1.1 นับ 47 ผิด เสาเหล็ก H250x175 จึงเป็น 46 ต้น)</t>
         </is>
       </c>
       <c r="D101" s="37" t="inlineStr"/>
@@ -9017,12 +9029,12 @@
       <c r="A102" s="37" t="inlineStr"/>
       <c r="B102" s="37" t="inlineStr">
         <is>
-          <t>โครงหลังคา</t>
+          <t>เหล็กเสริม</t>
         </is>
       </c>
       <c r="C102" s="37" t="inlineStr">
         <is>
-          <t>ยังไม่มีแบบโครงสร้างหลังคา น้ำหนักเหล็กโครงถัก/แป/ค้ำยันเป็นค่าประมาณจากโมเดล BIM</t>
+          <t>เหล็กเสริม คสล. ทุกรายการรอเอกสารการออกแบบเหล็กเสริมจากผู้ออกแบบ ตัวเลขในหมายเหตุเป็นค่าอ้างอิงเท่านั้น ไม่ใช้เป็นปริมาณ</t>
         </is>
       </c>
       <c r="D102" s="37" t="inlineStr"/>
@@ -9031,15 +9043,29 @@
       <c r="A103" s="37" t="inlineStr"/>
       <c r="B103" s="37" t="inlineStr">
         <is>
+          <t>โครงหลังคา</t>
+        </is>
+      </c>
+      <c r="C103" s="37" t="inlineStr">
+        <is>
+          <t>ยังไม่มีแบบโครงสร้างหลังคา น้ำหนักเหล็กโครงถัก/แป/ค้ำยันเป็นค่าประมาณจากโมเดล BIM</t>
+        </is>
+      </c>
+      <c r="D103" s="37" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="37" t="inlineStr"/>
+      <c r="B104" s="37" t="inlineStr">
+        <is>
           <t>ดินถม</t>
         </is>
       </c>
-      <c r="C103" s="37" t="inlineStr">
+      <c r="C104" s="37" t="inlineStr">
         <is>
           <t>ผู้ว่าจ้างยืนยัน 27/10/69: ดินเดิมอยู่ที่ ±0.00 (ระดับถนนรอบอาคาร) ระดับ -1.50 คือถนนสาธารณะ คิด BOQ ถมหนา 0.30 ม. ปริมาณจริงเบิกตามผลสำรวจระดับ P1.2</t>
         </is>
       </c>
-      <c r="D103" s="37" t="inlineStr"/>
+      <c r="D104" s="37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11451,7 +11477,7 @@
       <c r="A59" s="46" t="inlineStr"/>
       <c r="B59" s="46" t="inlineStr">
         <is>
-          <t>4.1.1: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S2 = 249) → รอผู้ว่าจ้างยืนยัน 249 (ตาราง S2) หรือ 232 (ผัง)</t>
+          <t>4.1.1: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S2 = 249) → ผู้ว่าจ้างยืนยัน 249 – ผังแสดง 232 ตำแหน่ง ขอตำแหน่ง 17 ต้นจากผู้ออกแบบ</t>
         </is>
       </c>
       <c r="C59" s="46" t="n"/>
@@ -11465,7 +11491,7 @@
       <c r="A60" s="46" t="inlineStr"/>
       <c r="B60" s="46" t="inlineStr">
         <is>
-          <t>4.1.2: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S1.1 = 249) → รอผู้ว่าจ้างยืนยัน 249 หรือ 232 ตาม 4.1.1</t>
+          <t>4.1.2: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S1.1 = 249) → ตาม 4.1.1 – ยอมรับ</t>
         </is>
       </c>
       <c r="C60" s="46" t="n"/>

</xml_diff>

<commit_message>
Add per-location structural schedule for footings, columns and beams
- every footing, column and beam span gets an ID tied to its grid
  position, shown in the viewer and IFC
- 02_ตารางโครงสร้าง workbook: size, levels, excavation depth, piles,
  concrete, formwork per footing; section, lengths, levels per beam span
  and column; rebar entry sheets with formulas for bars and stirrups
- transformer pad from A104, chemical room floor +0.40 from A103
- open issues sheet lists conflicts between A103/A104 and S201

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
+++ b/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. พร้อมขอบกั้นรั่วไหล</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 4.00x6.00 ม. พื้น +0.40 ผนัง W2 สูงถึง +3.30 จันทันเหล็ก C100x50x20x2.3 พร้อมขอบกั้นรั่วไหล</t>
         </is>
       </c>
       <c r="C31" s="27" t="n">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="K31" s="19" t="inlineStr">
         <is>
-          <t>เพิ่ม: A101</t>
+          <t>แบบ A103 (พื้น +0.40 และเสากลางผนังที่ y=3.0 ม. ไม่ตรงกับ S201/S6.1 ยืนยัน)</t>
         </is>
       </c>
     </row>
@@ -5872,20 +5872,20 @@
       <c r="K14" s="16" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>4.3.1</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
         </is>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="D15" s="25" t="inlineStr">
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>ต้น</t>
         </is>
@@ -5904,34 +5904,34 @@
         <f>F15+H15</f>
         <v/>
       </c>
-      <c r="J15" s="25" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+      <c r="J15" s="33" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>S2 / S201</t>
+          <t>S2 / S201 = 6 ต้น; A104 แสดง 3x3 = 9 ต้น (ยืนยัน)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>4.3.2</t>
         </is>
       </c>
-      <c r="B16" s="34" t="inlineStr">
-        <is>
-          <t>ฐานหม้อแปลง คสล. (ขนาดรอแบบขยาย)</t>
-        </is>
-      </c>
-      <c r="C16" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>ชุด</t>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>แท่นหม้อแปลง 750 kVA คสล.: ฐาน 5.00x3.00x0.40 ม. + แท่น 3.50x1.75x0.15 ม. (A104)</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>ลบ.ม.</t>
         </is>
       </c>
       <c r="E16" s="21" t="n"/>
@@ -5948,12 +5948,16 @@
         <f>F16+H16</f>
         <v/>
       </c>
-      <c r="J16" s="33" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
-        </is>
-      </c>
-      <c r="K16" s="19" t="inlineStr"/>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
+        </is>
+      </c>
+      <c r="K16" s="19" t="inlineStr">
+        <is>
+          <t>แบบ A104: คอนกรีต 6.00 + 0.92 ลบ.ม. ไม้แบบ 7.98 ตร.ม.; A104 แสดงเข็ม 9 ต้น แต่ S201 แสดง 6 ต้น (ยืนยัน)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -8354,12 +8358,12 @@
       </c>
       <c r="C68" s="37" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 21.84 ตร.ม. พร้อมขอบกั้นรั่วไหล</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 4.00x6.00 ม. พื้น +0.40 ผนัง W2 สูงถึง +3.30 จันทันเหล็ก C100x50x20x2.3 พร้อมขอบกั้นรั่วไหล</t>
         </is>
       </c>
       <c r="D68" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A101</t>
+          <t>แบบ A103 (พื้น +0.40 และเสากลางผนังที่ y=3.0 ม. ไม่ตรงกับ S201/S6.1 ยืนยัน)</t>
         </is>
       </c>
     </row>
@@ -8589,9 +8593,9 @@
           <t>4.3.1</t>
         </is>
       </c>
-      <c r="B79" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+      <c r="B79" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C79" s="37" t="inlineStr">
@@ -8601,7 +8605,7 @@
       </c>
       <c r="D79" s="37" t="inlineStr">
         <is>
-          <t>S2 / S201</t>
+          <t>S2 / S201 = 6 ต้น; A104 แสดง 3x3 = 9 ต้น (ยืนยัน)</t>
         </is>
       </c>
     </row>
@@ -8611,17 +8615,21 @@
           <t>4.3.2</t>
         </is>
       </c>
-      <c r="B80" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+      <c r="B80" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C80" s="37" t="inlineStr">
         <is>
-          <t>ฐานหม้อแปลง คสล. (ขนาดรอแบบขยาย)</t>
-        </is>
-      </c>
-      <c r="D80" s="37" t="inlineStr"/>
+          <t>แท่นหม้อแปลง 750 kVA คสล.: ฐาน 5.00x3.00x0.40 ม. + แท่น 3.50x1.75x0.15 ม. (A104)</t>
+        </is>
+      </c>
+      <c r="D80" s="37" t="inlineStr">
+        <is>
+          <t>แบบ A104: คอนกรีต 6.00 + 0.92 ลบ.ม. ไม้แบบ 7.98 ตร.ม.; A104 แสดงเข็ม 9 ต้น แต่ S201 แสดง 6 ต้น (ยืนยัน)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="37" t="inlineStr">
@@ -11131,10 +11139,10 @@
         </is>
       </c>
       <c r="E47" s="46" t="n">
-        <v>2389.58</v>
+        <v>2384.78</v>
       </c>
       <c r="F47" s="46" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="G47" s="48" t="inlineStr">
         <is>
@@ -11505,7 +11513,7 @@
       <c r="A61" s="46" t="inlineStr"/>
       <c r="B61" s="46" t="inlineStr">
         <is>
-          <t>4.1.3: BOQ 2,440.69 เทียบ 2,389.58 (+2.1%) – โมเดล (แนวเขต S202 หักอาคาร/ถัง/ทางลาด) → ใช้ตาราง S6.1 (ค่าออกแบบ) โมเดลใช้แนวเขตที่ดินร่นเข้า 0.6 ม. โดยประมาณ – ยอมรับ</t>
+          <t>4.1.3: BOQ 2,440.69 เทียบ 2,384.78 (+2.3%) – โมเดล (แนวเขต S202 หักอาคาร/ถัง/ทางลาด) → ใช้ตาราง S6.1 (ค่าออกแบบ) โมเดลใช้แนวเขตที่ดินร่นเข้า 0.6 ม. โดยประมาณ – ยอมรับ</t>
         </is>
       </c>
       <c r="C61" s="46" t="n"/>

</xml_diff>

<commit_message>
Add steel column base and top plates with anchor bolts
- base plate and top plate PL20x200x450 and 6 anchor bolts M20x750 per
  steel column, as given by the owner; grout 25 mm; bolts cast with the
  RC columns; steel column shaft shortened to 4.435 m
- detail D01 (plan and section) generated from model values, shown in
  the viewer and saved as SVG
- BOQ items 2.5.6-2.5.9 added, 2.5.1 and 2.5.4 recalculated
- schedule sheet 8 lists every joint and checks bolt-to-bar clearance
  from the column rebar entered in sheet 4

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018fTFw9DNpzgpK9RQnmJQ9j
</commit_message>
<xml_diff>
--- a/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
+++ b/tongcheng-bim/out/01_BOQ_งานหลัก_v2.xlsx
@@ -739,15 +739,15 @@
         </is>
       </c>
       <c r="C6" s="6">
-        <f>'2-งานโครงสร้าง'!F44</f>
+        <f>'2-งานโครงสร้าง'!F47</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>'2-งานโครงสร้าง'!H44</f>
+        <f>'2-งานโครงสร้าง'!H47</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>'2-งานโครงสร้าง'!I44</f>
+        <f>'2-งานโครงสร้าง'!I47</f>
         <v/>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -2390,7 +2390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3553,11 +3553,11 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>เสาเหล็ก H250x175x44.1 กก./ม. บนหัวเสา คสล. +4.50 ถึง +9.00 พร้อมแผ่นเหล็กฐาน Anchor bolt</t>
+          <t>เสาเหล็ก H244x175x7x11 (H250x175) 44.1 กก./ม. จากแผ่นเหล็กฐาน +4.545 ถึงใต้แผ่นหัวเสา +8.98</t>
         </is>
       </c>
       <c r="C32" s="24" t="n">
-        <v>9311</v>
+        <v>8997</v>
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
@@ -3585,7 +3585,7 @@
       </c>
       <c r="K32" s="19" t="inlineStr">
         <is>
-          <t>แก้ไข: 46 ต้น (ตาม F2P 46 ฐาน) x 4.59 ม. (215.72/47 จาก S4.1) = 211.13 ม. x 44.1 กก./ม.</t>
+          <t>แก้ไข: 46 ต้น x 4.435 ม. = 204.01 ม. x 44.1 กก./ม. (หักเกราท์ 25 + แผ่นเหล็ก 20+20 มม.)</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
         </is>
       </c>
       <c r="C35" s="35" t="n">
-        <v>5880</v>
+        <v>5849</v>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="K35" s="19" t="inlineStr">
         <is>
-          <t>แก้ไข: ค้ำยัน 303 + จุดต่อ 10% ของ 2.5.1-2.5.3 (55,773) = 5,880 กก. ประมาณการ รอแบบ</t>
+          <t>แก้ไข: ค้ำยัน 303 + จุดต่อ 10% ของ 2.5.1-2.5.3 (55,459) = 5,849 กก. ไม่รวมแผ่นเหล็กฐาน/หัวเสา (2.5.7-2.5.9) ประมาณการ รอแบบ</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) ใต้แผ่นฐานเสาเหล็ก</t>
+          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) หนา 25 มม. ใต้แผ่นเหล็กฐาน</t>
         </is>
       </c>
       <c r="C37" s="27" t="n">
@@ -3801,44 +3801,67 @@
       </c>
       <c r="K37" s="19" t="inlineStr">
         <is>
-          <t>เพิ่ม: เสาเหล็กบนหัวเสา คสล. C1 45 + C2 1 (S201)</t>
+          <t>เพิ่ม: เสาเหล็กบนหัวเสา คสล. C1 45 + C2 1 (S201) ขนาด 0.25x0.50 ม./จุด</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-      <c r="B38" s="16" t="inlineStr">
-        <is>
-          <t>หมวดงานชั้นลอย F8 (ระดับ +3.30)</t>
-        </is>
-      </c>
-      <c r="C38" s="17" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="17" t="n"/>
-      <c r="F38" s="17" t="n"/>
-      <c r="G38" s="17" t="n"/>
-      <c r="H38" s="17" t="n"/>
-      <c r="I38" s="17" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="16" t="n"/>
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>2.5.7</t>
+        </is>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>แผ่นเหล็กฐาน (Base plate) PL 20x200x450 มม. เจาะรู 6 รู เชื่อมกับเสาเหล็ก</t>
+        </is>
+      </c>
+      <c r="C38" s="27" t="n">
+        <v>649.98</v>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>กก.</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="n"/>
+      <c r="F38" s="20">
+        <f>IF(C38="",0,C38*E38)</f>
+        <v/>
+      </c>
+      <c r="G38" s="21" t="n"/>
+      <c r="H38" s="20">
+        <f>IF(C38="",0,C38*G38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="20">
+        <f>F38+H38</f>
+        <v/>
+      </c>
+      <c r="J38" s="25" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
+        </is>
+      </c>
+      <c r="K38" s="19" t="inlineStr">
+        <is>
+          <t>เพิ่ม: ผู้ว่าจ้างกำหนดเบื้องต้น 46 แผ่น x 14.13 กก. (แบบขยาย D01)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>2.6.1</t>
+          <t>2.5.8</t>
         </is>
       </c>
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
+          <t>แผ่นเหล็กหัวเสา (Top plate) PL 20x200x450 มม. ที่ +9.00 รับโครงถัก</t>
         </is>
       </c>
       <c r="C39" s="27" t="n">
-        <v>6703</v>
+        <v>649.98</v>
       </c>
       <c r="D39" s="25" t="inlineStr">
         <is>
@@ -3866,27 +3889,27 @@
       </c>
       <c r="K39" s="19" t="inlineStr">
         <is>
-          <t>เพิ่ม: S4.1 36 ต้น ยาว 100.80 ม.</t>
+          <t>เพิ่ม: ผู้ว่าจ้างกำหนดเบื้องต้น ขนาดเดียวกับแผ่นฐาน 46 แผ่น</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="33" t="inlineStr">
-        <is>
-          <t>2.6.2</t>
-        </is>
-      </c>
-      <c r="B40" s="34" t="inlineStr">
-        <is>
-          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
-        </is>
-      </c>
-      <c r="C40" s="35" t="n">
-        <v>5219</v>
-      </c>
-      <c r="D40" s="33" t="inlineStr">
-        <is>
-          <t>กก.</t>
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>2.5.9</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Anchor bolt M20 ยาว 750 มม. ปลายงอ พร้อมแป้นเกลียว 2 ตัว แหวน และแบบจับตำแหน่ง (Template) ฝังในหัวเสา คสล.</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="n">
+        <v>276</v>
+      </c>
+      <c r="D40" s="25" t="inlineStr">
+        <is>
+          <t>ชุด</t>
         </is>
       </c>
       <c r="E40" s="21" t="n"/>
@@ -3903,78 +3926,55 @@
         <f>F40+H40</f>
         <v/>
       </c>
-      <c r="J40" s="33" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+      <c r="J40" s="25" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="K40" s="19" t="inlineStr">
         <is>
-          <t>เพิ่ม: ประมาณการ H200x100 ตารางคาน 3.00 ม.</t>
+          <t>เพิ่ม: 6 ชุด/เสา x 46 ต้น (~2.01 กก./ชุด) ติดตั้งก่อนเทเสา คสล.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="25" t="inlineStr">
-        <is>
-          <t>2.6.3</t>
-        </is>
-      </c>
-      <c r="B41" s="26" t="inlineStr">
-        <is>
-          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
-        </is>
-      </c>
-      <c r="C41" s="27" t="n">
-        <v>306.15</v>
-      </c>
-      <c r="D41" s="25" t="inlineStr">
-        <is>
-          <t>ตร.ม.</t>
-        </is>
-      </c>
-      <c r="E41" s="21" t="n"/>
-      <c r="F41" s="20">
-        <f>IF(C41="",0,C41*E41)</f>
-        <v/>
-      </c>
-      <c r="G41" s="21" t="n"/>
-      <c r="H41" s="20">
-        <f>IF(C41="",0,C41*G41)</f>
-        <v/>
-      </c>
-      <c r="I41" s="20">
-        <f>F41+H41</f>
-        <v/>
-      </c>
-      <c r="J41" s="25" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
-        </is>
-      </c>
-      <c r="K41" s="19" t="inlineStr">
-        <is>
-          <t>เพิ่ม: S6.1 306.15 ตร.ม.</t>
-        </is>
-      </c>
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>หมวดงานชั้นลอย F8 (ระดับ +3.30)</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="17" t="n"/>
+      <c r="G41" s="17" t="n"/>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="17" t="n"/>
+      <c r="J41" s="15" t="n"/>
+      <c r="K41" s="16" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="25" t="inlineStr">
         <is>
-          <t>2.6.4</t>
+          <t>2.6.1</t>
         </is>
       </c>
       <c r="B42" s="26" t="inlineStr">
         <is>
-          <t>บันไดเหล็กขึ้นชั้นลอย กว้าง ~1.40 ม. พร้อมราวกันตก</t>
+          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
         </is>
       </c>
       <c r="C42" s="27" t="n">
-        <v>1</v>
+        <v>6703</v>
       </c>
       <c r="D42" s="25" t="inlineStr">
         <is>
-          <t>ชุด</t>
+          <t>กก.</t>
         </is>
       </c>
       <c r="E42" s="21" t="n"/>
@@ -3998,27 +3998,27 @@
       </c>
       <c r="K42" s="19" t="inlineStr">
         <is>
-          <t>เพิ่ม: ตำแหน่ง DN แนวกริด D</t>
+          <t>เพิ่ม: S4.1 36 ต้น ยาว 100.80 ม.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="25" t="inlineStr">
-        <is>
-          <t>2.6.5</t>
-        </is>
-      </c>
-      <c r="B43" s="26" t="inlineStr">
-        <is>
-          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
-        </is>
-      </c>
-      <c r="C43" s="27" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="D43" s="25" t="inlineStr">
-        <is>
-          <t>ม.</t>
+      <c r="A43" s="33" t="inlineStr">
+        <is>
+          <t>2.6.2</t>
+        </is>
+      </c>
+      <c r="B43" s="34" t="inlineStr">
+        <is>
+          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="n">
+        <v>5219</v>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>กก.</t>
         </is>
       </c>
       <c r="E43" s="21" t="n"/>
@@ -4035,45 +4035,177 @@
         <f>F43+H43</f>
         <v/>
       </c>
-      <c r="J43" s="25" t="inlineStr">
+      <c r="J43" s="33" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
+        </is>
+      </c>
+      <c r="K43" s="19" t="inlineStr">
+        <is>
+          <t>เพิ่ม: ประมาณการ H200x100 ตารางคาน 3.00 ม.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>2.6.3</t>
+        </is>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
+        </is>
+      </c>
+      <c r="C44" s="27" t="n">
+        <v>306.15</v>
+      </c>
+      <c r="D44" s="25" t="inlineStr">
+        <is>
+          <t>ตร.ม.</t>
+        </is>
+      </c>
+      <c r="E44" s="21" t="n"/>
+      <c r="F44" s="20">
+        <f>IF(C44="",0,C44*E44)</f>
+        <v/>
+      </c>
+      <c r="G44" s="21" t="n"/>
+      <c r="H44" s="20">
+        <f>IF(C44="",0,C44*G44)</f>
+        <v/>
+      </c>
+      <c r="I44" s="20">
+        <f>F44+H44</f>
+        <v/>
+      </c>
+      <c r="J44" s="25" t="inlineStr">
         <is>
           <t>เพิ่มใหม่</t>
         </is>
       </c>
-      <c r="K43" s="19" t="inlineStr">
+      <c r="K44" s="19" t="inlineStr">
+        <is>
+          <t>เพิ่ม: S6.1 306.15 ตร.ม.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="25" t="inlineStr">
+        <is>
+          <t>2.6.4</t>
+        </is>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>บันไดเหล็กขึ้นชั้นลอย กว้าง ~1.40 ม. พร้อมราวกันตก</t>
+        </is>
+      </c>
+      <c r="C45" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="25" t="inlineStr">
+        <is>
+          <t>ชุด</t>
+        </is>
+      </c>
+      <c r="E45" s="21" t="n"/>
+      <c r="F45" s="20">
+        <f>IF(C45="",0,C45*E45)</f>
+        <v/>
+      </c>
+      <c r="G45" s="21" t="n"/>
+      <c r="H45" s="20">
+        <f>IF(C45="",0,C45*G45)</f>
+        <v/>
+      </c>
+      <c r="I45" s="20">
+        <f>F45+H45</f>
+        <v/>
+      </c>
+      <c r="J45" s="25" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
+        </is>
+      </c>
+      <c r="K45" s="19" t="inlineStr">
+        <is>
+          <t>เพิ่ม: ตำแหน่ง DN แนวกริด D</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>2.6.5</t>
+        </is>
+      </c>
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
+        </is>
+      </c>
+      <c r="C46" s="27" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="D46" s="25" t="inlineStr">
+        <is>
+          <t>ม.</t>
+        </is>
+      </c>
+      <c r="E46" s="21" t="n"/>
+      <c r="F46" s="20">
+        <f>IF(C46="",0,C46*E46)</f>
+        <v/>
+      </c>
+      <c r="G46" s="21" t="n"/>
+      <c r="H46" s="20">
+        <f>IF(C46="",0,C46*G46)</f>
+        <v/>
+      </c>
+      <c r="I46" s="20">
+        <f>F46+H46</f>
+        <v/>
+      </c>
+      <c r="J46" s="25" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
+        </is>
+      </c>
+      <c r="K46" s="19" t="inlineStr">
         <is>
           <t>เพิ่ม: ขอบด้านเปิด 18 + 17 ม. หักช่องบันได 1.40 ม.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="28" t="n"/>
-      <c r="B44" s="10" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="28" t="n"/>
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>รวมหมวดที่ 2 งานโครงสร้าง</t>
         </is>
       </c>
-      <c r="C44" s="29" t="n"/>
-      <c r="D44" s="28" t="n"/>
-      <c r="E44" s="29" t="n"/>
-      <c r="F44" s="30">
-        <f>SUM(F5:F43)</f>
-        <v/>
-      </c>
-      <c r="G44" s="29" t="n"/>
-      <c r="H44" s="30">
-        <f>SUM(H5:H43)</f>
-        <v/>
-      </c>
-      <c r="I44" s="30">
-        <f>SUM(I5:I43)</f>
-        <v/>
-      </c>
-      <c r="J44" s="28" t="n"/>
-      <c r="K44" s="31" t="n"/>
-    </row>
-    <row r="45">
-      <c r="B45" s="32" t="inlineStr">
+      <c r="C47" s="29" t="n"/>
+      <c r="D47" s="28" t="n"/>
+      <c r="E47" s="29" t="n"/>
+      <c r="F47" s="30">
+        <f>SUM(F5:F46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="29" t="n"/>
+      <c r="H47" s="30">
+        <f>SUM(H5:H46)</f>
+        <v/>
+      </c>
+      <c r="I47" s="30">
+        <f>SUM(I5:I46)</f>
+        <v/>
+      </c>
+      <c r="J47" s="28" t="n"/>
+      <c r="K47" s="31" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="32" t="inlineStr">
         <is>
           <t>หมายเหตุ: ช่องสีเหลืองสำหรับกรอกราคาต่อหน่วย | สีแดง = เพิ่มใหม่ | สีส้ม = แก้ไขปริมาณ/รายละเอียด | สีม่วง = รอข้อมูล/ยืนยันจากผู้ออกแบบ</t>
         </is>
@@ -6881,7 +7013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D104"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7680,12 +7812,12 @@
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
-          <t>เสาเหล็ก H250x175x44.1 กก./ม. บนหัวเสา คสล. +4.50 ถึง +9.00 พร้อมแผ่นเหล็กฐาน Anchor bolt</t>
+          <t>เสาเหล็ก H244x175x7x11 (H250x175) 44.1 กก./ม. จากแผ่นเหล็กฐาน +4.545 ถึงใต้แผ่นหัวเสา +8.98</t>
         </is>
       </c>
       <c r="D37" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: 46 ต้น (ตาม F2P 46 ฐาน) x 4.59 ม. (215.72/47 จาก S4.1) = 211.13 ม. x 44.1 กก./ม.</t>
+          <t>แก้ไข: 46 ต้น x 4.435 ม. = 204.01 ม. x 44.1 กก./ม. (หักเกราท์ 25 + แผ่นเหล็ก 20+20 มม.)</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7883,7 @@
       </c>
       <c r="D40" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: ค้ำยัน 303 + จุดต่อ 10% ของ 2.5.1-2.5.3 (55,773) = 5,880 กก. ประมาณการ รอแบบ</t>
+          <t>แก้ไข: ค้ำยัน 303 + จุดต่อ 10% ของ 2.5.1-2.5.3 (55,459) = 5,849 กก. ไม่รวมแผ่นเหล็กฐาน/หัวเสา (2.5.7-2.5.9) ประมาณการ รอแบบ</t>
         </is>
       </c>
     </row>
@@ -7786,19 +7918,19 @@
       </c>
       <c r="C42" s="37" t="inlineStr">
         <is>
-          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) ใต้แผ่นฐานเสาเหล็ก</t>
+          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) หนา 25 มม. ใต้แผ่นเหล็กฐาน</t>
         </is>
       </c>
       <c r="D42" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: เสาเหล็กบนหัวเสา คสล. C1 45 + C2 1 (S201)</t>
+          <t>เพิ่ม: เสาเหล็กบนหัวเสา คสล. C1 45 + C2 1 (S201) ขนาด 0.25x0.50 ม./จุด</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="37" t="inlineStr">
         <is>
-          <t>2.6.1</t>
+          <t>2.5.7</t>
         </is>
       </c>
       <c r="B43" s="39" t="inlineStr">
@@ -7808,41 +7940,41 @@
       </c>
       <c r="C43" s="37" t="inlineStr">
         <is>
-          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
+          <t>แผ่นเหล็กฐาน (Base plate) PL 20x200x450 มม. เจาะรู 6 รู เชื่อมกับเสาเหล็ก</t>
         </is>
       </c>
       <c r="D43" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: S4.1 36 ต้น ยาว 100.80 ม.</t>
+          <t>เพิ่ม: ผู้ว่าจ้างกำหนดเบื้องต้น 46 แผ่น x 14.13 กก. (แบบขยาย D01)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="37" t="inlineStr">
         <is>
-          <t>2.6.2</t>
-        </is>
-      </c>
-      <c r="B44" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>2.5.8</t>
+        </is>
+      </c>
+      <c r="B44" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C44" s="37" t="inlineStr">
         <is>
-          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
+          <t>แผ่นเหล็กหัวเสา (Top plate) PL 20x200x450 มม. ที่ +9.00 รับโครงถัก</t>
         </is>
       </c>
       <c r="D44" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ประมาณการ H200x100 ตารางคาน 3.00 ม.</t>
+          <t>เพิ่ม: ผู้ว่าจ้างกำหนดเบื้องต้น ขนาดเดียวกับแผ่นฐาน 46 แผ่น</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="37" t="inlineStr">
         <is>
-          <t>2.6.3</t>
+          <t>2.5.9</t>
         </is>
       </c>
       <c r="B45" s="39" t="inlineStr">
@@ -7852,19 +7984,19 @@
       </c>
       <c r="C45" s="37" t="inlineStr">
         <is>
-          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
+          <t>Anchor bolt M20 ยาว 750 มม. ปลายงอ พร้อมแป้นเกลียว 2 ตัว แหวน และแบบจับตำแหน่ง (Template) ฝังในหัวเสา คสล.</t>
         </is>
       </c>
       <c r="D45" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: S6.1 306.15 ตร.ม.</t>
+          <t>เพิ่ม: 6 ชุด/เสา x 46 ต้น (~2.01 กก./ชุด) ติดตั้งก่อนเทเสา คสล.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="37" t="inlineStr">
         <is>
-          <t>2.6.4</t>
+          <t>2.6.1</t>
         </is>
       </c>
       <c r="B46" s="39" t="inlineStr">
@@ -7874,41 +8006,41 @@
       </c>
       <c r="C46" s="37" t="inlineStr">
         <is>
-          <t>บันไดเหล็กขึ้นชั้นลอย กว้าง ~1.40 ม. พร้อมราวกันตก</t>
+          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
         </is>
       </c>
       <c r="D46" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ตำแหน่ง DN แนวกริด D</t>
+          <t>เพิ่ม: S4.1 36 ต้น ยาว 100.80 ม.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="37" t="inlineStr">
         <is>
-          <t>2.6.5</t>
-        </is>
-      </c>
-      <c r="B47" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>2.6.2</t>
+        </is>
+      </c>
+      <c r="B47" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C47" s="37" t="inlineStr">
         <is>
-          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
+          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
         </is>
       </c>
       <c r="D47" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ขอบด้านเปิด 18 + 17 ม. หักช่องบันได 1.40 ม.</t>
+          <t>เพิ่ม: ประมาณการ H200x100 ตารางคาน 3.00 ม.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="37" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>2.6.3</t>
         </is>
       </c>
       <c r="B48" s="39" t="inlineStr">
@@ -7918,19 +8050,19 @@
       </c>
       <c r="C48" s="37" t="inlineStr">
         <is>
-          <t>หลังคาเมทัลชีทหนา 0.47 มม. พร้อมฉนวน PU 25 มม. (พื้นที่ตามลาด)</t>
+          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
         </is>
       </c>
       <c r="D48" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: จากโมเดล 2 ลาด 30.2 ม. x 55 ม. (สเปควัสดุรอยืนยัน)</t>
+          <t>เพิ่ม: S6.1 306.15 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="37" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>2.6.4</t>
         </is>
       </c>
       <c r="B49" s="39" t="inlineStr">
@@ -7940,19 +8072,19 @@
       </c>
       <c r="C49" s="37" t="inlineStr">
         <is>
-          <t>Jack roof กว้าง 6.00 ม. ยาว 42.00 ม. สัน +15.25 พร้อมตะแกรงระบายอากาศ</t>
+          <t>บันไดเหล็กขึ้นชั้นลอย กว้าง ~1.40 ม. พร้อมราวกันตก</t>
         </is>
       </c>
       <c r="D49" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A202</t>
+          <t>เพิ่ม: ตำแหน่ง DN แนวกริด D</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>2.6.5</t>
         </is>
       </c>
       <c r="B50" s="39" t="inlineStr">
@@ -7962,19 +8094,19 @@
       </c>
       <c r="C50" s="37" t="inlineStr">
         <is>
-          <t>ครอบสัน ครอบข้าง แผ่นปิดเชิงชาย Flashing</t>
+          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
         </is>
       </c>
       <c r="D50" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม</t>
+          <t>เพิ่ม: ขอบด้านเปิด 18 + 17 ม. หักช่องบันได 1.40 ม.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="37" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="B51" s="39" t="inlineStr">
@@ -7984,41 +8116,41 @@
       </c>
       <c r="C51" s="37" t="inlineStr">
         <is>
-          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30 ม.</t>
+          <t>หลังคาเมทัลชีทหนา 0.47 มม. พร้อมฉนวน PU 25 มม. (พื้นที่ตามลาด)</t>
         </is>
       </c>
       <c r="D51" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ชายคาแนวกริด 1 และ 11</t>
+          <t>เพิ่ม: จากโมเดล 2 ลาด 30.2 ม. x 55 ม. (สเปควัสดุรอยืนยัน)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="37" t="inlineStr">
         <is>
-          <t>3.1.5</t>
-        </is>
-      </c>
-      <c r="B52" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.1.2</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C52" s="37" t="inlineStr">
         <is>
-          <t>ท่อระบายน้ำฝน PVC Ø4" พร้อมอุปกรณ์ยึด</t>
+          <t>Jack roof กว้าง 6.00 ม. ยาว 42.00 ม. สัน +15.25 พร้อมตะแกรงระบายอากาศ</t>
         </is>
       </c>
       <c r="D52" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: 10 จุด x 10 ม. (สมมติ)</t>
+          <t>เพิ่ม: A202</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
-          <t>3.1.6</t>
+          <t>3.1.3</t>
         </is>
       </c>
       <c r="B53" s="39" t="inlineStr">
@@ -8028,173 +8160,173 @@
       </c>
       <c r="C53" s="37" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท ระดับ +5.20 ถึงชายคา/จั่ว</t>
+          <t>ครอบสัน ครอบข้าง แผ่นปิดเชิงชาย Flashing</t>
         </is>
       </c>
       <c r="D53" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: จากโมเดล ตาม A202</t>
+          <t>เพิ่ม</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="37" t="inlineStr">
         <is>
-          <t>3.1.7</t>
-        </is>
-      </c>
-      <c r="B54" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.1.4</t>
+        </is>
+      </c>
+      <c r="B54" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C54" s="37" t="inlineStr">
         <is>
-          <t>ตะแกรงกันนก/ช่องระบายอากาศ ระดับ +4.50 ถึง +5.20 รอบอาคาร</t>
+          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30 ม.</t>
         </is>
       </c>
       <c r="D54" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ช่องระหว่างผนังก่อกับเมทัลชีท (A202) หักประตูม้วน 12 ม.</t>
+          <t>เพิ่ม: ชายคาแนวกริด 1 และ 11</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="37" t="inlineStr">
         <is>
-          <t>3.2.1</t>
-        </is>
-      </c>
-      <c r="B55" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>3.1.5</t>
+        </is>
+      </c>
+      <c r="B55" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C55" s="37" t="inlineStr">
         <is>
-          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ม. +0.50 ถึง +4.35 (ต่ำกว่าหัวเสา คสล. 0.15 ม.)</t>
+          <t>ท่อระบายน้ำฝน PVC Ø4" พร้อมอุปกรณ์ยึด</t>
         </is>
       </c>
       <c r="D55" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: ผนัง 36 ช่วง ยาวสุทธิ 205.20 ม. x 3.85 ม. หักประตู D1 2 ช่อง, เสาเอ็น, คานเอ็น (ดูชีต 'ผนัง-รายละเอียด')</t>
+          <t>เพิ่ม: 10 จุด x 10 ม. (สมมติ)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="37" t="inlineStr">
         <is>
-          <t>3.2.2</t>
-        </is>
-      </c>
-      <c r="B56" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>3.1.6</t>
+        </is>
+      </c>
+      <c r="B56" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C56" s="37" t="inlineStr">
         <is>
-          <t>ฉาบปูนผนังก่อ คานเอ็น คานทับหลัง และเสาเอ็น 2 ด้าน (+0.50 ถึง +4.50)</t>
+          <t>ผนังเมทัลชีท ระดับ +5.20 ถึงชายคา/จั่ว</t>
         </is>
       </c>
       <c r="D56" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: 205.20 ม. x 4.00 ม. x 2 ด้าน หักประตู D1</t>
+          <t>เพิ่ม: จากโมเดล ตาม A202</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="37" t="inlineStr">
         <is>
-          <t>3.2.3</t>
-        </is>
-      </c>
-      <c r="B57" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.1.7</t>
+        </is>
+      </c>
+      <c r="B57" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C57" s="37" t="inlineStr">
         <is>
-          <t>คานทับหลัง คสล. 0.15x0.15 ม. ระดับ +4.35 ถึง +4.50 (คอนกรีต ไม้แบบ)</t>
+          <t>ตะแกรงกันนก/ช่องระบายอากาศ ระดับ +4.50 ถึง +5.20 รอบอาคาร</t>
         </is>
       </c>
       <c r="D57" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ผู้ว่าจ้างกำหนด คอนกรีต 4.62 ลบ.ม. ไม้แบบ 61.56 ตร.ม.</t>
+          <t>เพิ่ม: ช่องระหว่างผนังก่อกับเมทัลชีท (A202) หักประตูม้วน 12 ม.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="37" t="inlineStr">
         <is>
-          <t>3.2.4</t>
-        </is>
-      </c>
-      <c r="B58" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.2.1</t>
+        </is>
+      </c>
+      <c r="B58" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C58" s="37" t="inlineStr">
         <is>
-          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังวงกบประตู +2.60 (คอนกรีต ไม้แบบ)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ม. +0.50 ถึง +4.35 (ต่ำกว่าหัวเสา คสล. 0.15 ม.)</t>
         </is>
       </c>
       <c r="D58" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ผนังสูง 3.85 ม. &gt; 3 ม. ต้องมีคานเอ็นกลางผนัง คอนกรีต 3.08 ลบ.ม. ไม้แบบ 41.04 ตร.ม.</t>
+          <t>แก้ไข: ผนัง 36 ช่วง ยาวสุทธิ 205.20 ม. x 3.85 ม. หักประตู D1 2 ช่อง, เสาเอ็น, คานเอ็น (ดูชีต 'ผนัง-รายละเอียด')</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="37" t="inlineStr">
         <is>
-          <t>3.2.5</t>
-        </is>
-      </c>
-      <c r="B59" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.2.2</t>
+        </is>
+      </c>
+      <c r="B59" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C59" s="37" t="inlineStr">
         <is>
-          <t>เสาเอ็น คสล. 0.15x0.10 ม. สูง 3.85 ม. (กลางช่วงเสา 6 ม. และข้างวงกบประตู)</t>
+          <t>ฉาบปูนผนังก่อ คานเอ็น คานทับหลัง และเสาเอ็น 2 ด้าน (+0.50 ถึง +4.50)</t>
         </is>
       </c>
       <c r="D59" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ยาวรวม 146.30 ม. คอนกรีต 2.19 ลบ.ม. ไม้แบบ 29.26 ตร.ม.</t>
+          <t>แก้ไข: 205.20 ม. x 4.00 ม. x 2 ด้าน หักประตู D1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="37" t="inlineStr">
         <is>
-          <t>3.2.6</t>
-        </is>
-      </c>
-      <c r="B60" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.2.3</t>
+        </is>
+      </c>
+      <c r="B60" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C60" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริมคานทับหลัง คานเอ็น เสาเอ็น</t>
+          <t>คานทับหลัง คสล. 0.15x0.15 ม. ระดับ +4.35 ถึง +4.50 (คอนกรีต ไม้แบบ)</t>
         </is>
       </c>
       <c r="D60" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม</t>
+          <t>เพิ่ม: ผู้ว่าจ้างกำหนด คอนกรีต 4.62 ลบ.ม. ไม้แบบ 61.56 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="37" t="inlineStr">
         <is>
-          <t>3.2.7</t>
+          <t>3.2.4</t>
         </is>
       </c>
       <c r="B61" s="39" t="inlineStr">
@@ -8204,19 +8336,19 @@
       </c>
       <c r="C61" s="37" t="inlineStr">
         <is>
-          <t>ฉาบปูนเสา คสล. C1/C2 ที่ผิวเปิด (+0.50 ถึง +4.50)</t>
+          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังวงกบประตู +2.60 (คอนกรีต ไม้แบบ)</t>
         </is>
       </c>
       <c r="D61" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: เสาแนวผนัง 38 ต้น x 1.30 ม. + เสากลางอาคาร 8 ต้น x 1.60 ม. x สูง 4.00 ม.</t>
+          <t>เพิ่ม: ผนังสูง 3.85 ม. &gt; 3 ม. ต้องมีคานเอ็นกลางผนัง คอนกรีต 3.08 ลบ.ม. ไม้แบบ 41.04 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="37" t="inlineStr">
         <is>
-          <t>3.2.8</t>
+          <t>3.2.5</t>
         </is>
       </c>
       <c r="B62" s="39" t="inlineStr">
@@ -8226,195 +8358,195 @@
       </c>
       <c r="C62" s="37" t="inlineStr">
         <is>
-          <t>จับเซี้ยมมุมเสา คสล. มุมผนัง ขอบคานทับหลัง และขอบช่องประตู ก่อนฉาบเสาและผนัง</t>
+          <t>เสาเอ็น คสล. 0.15x0.10 ม. สูง 3.85 ม. (กลางช่วงเสา 6 ม. และข้างวงกบประตู)</t>
         </is>
       </c>
       <c r="D62" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: มุมเสาแนวผนัง 608.0 + มุมเสากลางอาคาร 128.0 + ขอบบนคานทับหลัง 2 ด้าน 410.4 + ขอบช่องประตู D1 20.8 ม.</t>
+          <t>เพิ่ม: ยาวรวม 146.30 ม. คอนกรีต 2.19 ลบ.ม. ไม้แบบ 29.26 ตร.ม.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="37" t="inlineStr">
         <is>
-          <t>3.3.1</t>
-        </is>
-      </c>
-      <c r="B63" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>3.2.6</t>
+        </is>
+      </c>
+      <c r="B63" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C63" s="37" t="inlineStr">
         <is>
-          <t>พื้นขัดมันผสม Floor Hardener</t>
+          <t>เหล็กเสริมคานทับหลัง คานเอ็น เสาเอ็น</t>
         </is>
       </c>
       <c r="D63" s="37" t="inlineStr">
         <is>
-          <t>เดิม 3,240 → พื้นที่ S1 (S6.1)</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="37" t="inlineStr">
         <is>
-          <t>3.4.1</t>
-        </is>
-      </c>
-      <c r="B64" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.2.7</t>
+        </is>
+      </c>
+      <c r="B64" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C64" s="37" t="inlineStr">
         <is>
-          <t>ประตูม้วนเหล็กไฟฟ้า ~6.00x4.00 ม. ทางลาดขนส่ง</t>
+          <t>ฉาบปูนเสา คสล. C1/C2 ที่ผิวเปิด (+0.50 ถึง +4.50)</t>
         </is>
       </c>
       <c r="D64" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ตำแหน่งตาม A101 ขนาดรอยืนยัน</t>
+          <t>เพิ่ม: เสาแนวผนัง 38 ต้น x 1.30 ม. + เสากลางอาคาร 8 ต้น x 1.60 ม. x สูง 4.00 ม.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="37" t="inlineStr">
         <is>
-          <t>3.4.2</t>
-        </is>
-      </c>
-      <c r="B65" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.2.8</t>
+        </is>
+      </c>
+      <c r="B65" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C65" s="37" t="inlineStr">
         <is>
-          <t>ประตู D1/D2/D4 และหน้าต่าง ตามแบบ A101</t>
+          <t>จับเซี้ยมมุมเสา คสล. มุมผนัง ขอบคานทับหลัง และขอบช่องประตู ก่อนฉาบเสาและผนัง</t>
         </is>
       </c>
       <c r="D65" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: รอตารางประตู-หน้าต่าง</t>
+          <t>เพิ่ม: มุมเสาแนวผนัง 608.0 + มุมเสากลางอาคาร 128.0 + ขอบบนคานทับหลัง 2 ด้าน 410.4 + ขอบช่องประตู D1 20.8 ม.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t>3.5.1</t>
-        </is>
-      </c>
-      <c r="B66" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.3.1</t>
+        </is>
+      </c>
+      <c r="B66" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C66" s="37" t="inlineStr">
         <is>
-          <t>ทาสีผนังและเสา ภายใน-ภายนอก (รองพื้น + ทับหน้า 2 เที่ยว)</t>
+          <t>พื้นขัดมันผสม Floor Hardener</t>
         </is>
       </c>
       <c r="D66" s="37" t="inlineStr">
         <is>
-          <t>แก้ไข: เท่ากับพื้นที่ฉาบ 3.2.2 + 3.2.7</t>
+          <t>เดิม 3,240 → พื้นที่ S1 (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="37" t="inlineStr">
         <is>
-          <t>3.6.1</t>
-        </is>
-      </c>
-      <c r="B67" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.4.1</t>
+        </is>
+      </c>
+      <c r="B67" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C67" s="37" t="inlineStr">
         <is>
-          <t>ห้อง MDB 17.79 ตร.ม. (ผนัง ประตูกันไฟ พื้น ฝ้า)</t>
+          <t>ประตูม้วนเหล็กไฟฟ้า ~6.00x4.00 ม. ทางลาดขนส่ง</t>
         </is>
       </c>
       <c r="D67" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A101</t>
+          <t>เพิ่ม: ตำแหน่งตาม A101 ขนาดรอยืนยัน</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="37" t="inlineStr">
         <is>
-          <t>3.6.2</t>
-        </is>
-      </c>
-      <c r="B68" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.4.2</t>
+        </is>
+      </c>
+      <c r="B68" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C68" s="37" t="inlineStr">
         <is>
-          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 4.00x6.00 ม. พื้น +0.40 ผนัง W2 สูงถึง +3.30 จันทันเหล็ก C100x50x20x2.3 พร้อมขอบกั้นรั่วไหล</t>
+          <t>ประตู D1/D2/D4 และหน้าต่าง ตามแบบ A101</t>
         </is>
       </c>
       <c r="D68" s="37" t="inlineStr">
         <is>
-          <t>แบบ A103 (พื้น +0.40 และเสากลางผนังที่ y=3.0 ม. ไม่ตรงกับ S201/S6.1 ยืนยัน)</t>
+          <t>เพิ่ม: รอตารางประตู-หน้าต่าง</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="37" t="inlineStr">
         <is>
-          <t>3.6.3</t>
-        </is>
-      </c>
-      <c r="B69" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.5.1</t>
+        </is>
+      </c>
+      <c r="B69" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C69" s="37" t="inlineStr">
         <is>
-          <t>อาคารห้องน้ำ 2.40 x 8.00 ม. (สุขภัณฑ์ กระเบื้อง ระบบสุขาภิบาลภายใน)</t>
+          <t>ทาสีผนังและเสา ภายใน-ภายนอก (รองพื้น + ทับหน้า 2 เที่ยว)</t>
         </is>
       </c>
       <c r="D69" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: A101/S201 รอแบบสถาปัตย์</t>
+          <t>แก้ไข: เท่ากับพื้นที่ฉาบ 3.2.2 + 3.2.7</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="37" t="inlineStr">
         <is>
-          <t>3.6.4</t>
-        </is>
-      </c>
-      <c r="B70" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>3.6.1</t>
+        </is>
+      </c>
+      <c r="B70" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C70" s="37" t="inlineStr">
         <is>
-          <t>ห้องประกอบแนวกริด A (กริด 8-10)</t>
+          <t>ห้อง MDB 17.79 ตร.ม. (ผนัง ประตูกันไฟ พื้น ฝ้า)</t>
         </is>
       </c>
       <c r="D70" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: เห็นในผัง A101 รอแบบ</t>
+          <t>เพิ่ม: A101</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="37" t="inlineStr">
         <is>
-          <t>3.6.5</t>
+          <t>3.6.2</t>
         </is>
       </c>
       <c r="B71" s="39" t="inlineStr">
@@ -8424,63 +8556,63 @@
       </c>
       <c r="C71" s="37" t="inlineStr">
         <is>
-          <t>บันได/ชานพัก คสล. หน้าประตู D1 ภายนอก (พื้น +0.50 ถนน ±0.00)</t>
+          <t>ห้องเก็บสารเคมี (Chemical Drum Storage) 4.00x6.00 ม. พื้น +0.40 ผนัง W2 สูงถึง +3.30 จันทันเหล็ก C100x50x20x2.3 พร้อมขอบกั้นรั่วไหล</t>
         </is>
       </c>
       <c r="D71" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ประตู D1 ผนังแนวกริด 1 และ 11 (A101) ระดับต่างกัน 0.50 ม.</t>
+          <t>แบบ A103 (พื้น +0.40 และเสากลางผนังที่ y=3.0 ม. ไม่ตรงกับ S201/S6.1 ยืนยัน)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="37" t="inlineStr">
         <is>
-          <t>4.1.1</t>
-        </is>
-      </c>
-      <c r="B72" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.6.3</t>
+        </is>
+      </c>
+      <c r="B72" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C72" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับพื้นถนนรอบอาคาร (I22-22) รวมค่าตอก</t>
+          <t>อาคารห้องน้ำ 2.40 x 8.00 ม. (สุขภัณฑ์ กระเบื้อง ระบบสุขาภิบาลภายใน)</t>
         </is>
       </c>
       <c r="D72" s="37" t="inlineStr">
         <is>
-          <t>กลุ่มเข็มถนน: ผู้ว่าจ้างยืนยัน 249 ต้น (ผัง S201/S202 แสดงตำแหน่ง 232 ต้น ขอตำแหน่งอีก 17 ต้นจากผู้ออกแบบ)</t>
+          <t>เพิ่ม: A101/S201 รอแบบสถาปัตย์</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="37" t="inlineStr">
         <is>
-          <t>4.1.2</t>
-        </is>
-      </c>
-      <c r="B73" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>3.6.4</t>
+        </is>
+      </c>
+      <c r="B73" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C73" s="37" t="inlineStr">
         <is>
-          <t>ฐาน F1A 0.60x0.60x0.30 ม. รับพื้นถนน</t>
+          <t>ห้องประกอบแนวกริด A (กริด 8-10)</t>
         </is>
       </c>
       <c r="D73" s="37" t="inlineStr">
         <is>
-          <t>ตามเข็มถนน 249 ต้น คอนกรีต 26.78, ทราย 35.86, คอนกรีตหยาบ 6.10 ลบ.ม. (S1.1)</t>
+          <t>เพิ่ม: เห็นในผัง A101 รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="37" t="inlineStr">
         <is>
-          <t>4.1.3</t>
+          <t>3.6.5</t>
         </is>
       </c>
       <c r="B74" s="39" t="inlineStr">
@@ -8490,19 +8622,19 @@
       </c>
       <c r="C74" s="37" t="inlineStr">
         <is>
-          <t>พื้นถนน S2 คสล. หนา 0.15 ม. TOP ±0.00 พร้อมรอยต่อ/ตัดรอยต่อ</t>
+          <t>บันได/ชานพัก คสล. หน้าประตู D1 ภายนอก (พื้น +0.50 ถนน ±0.00)</t>
         </is>
       </c>
       <c r="D74" s="37" t="inlineStr">
         <is>
-          <t>คอนกรีต 366.10 ลบ.ม. (S6.1)</t>
+          <t>เพิ่ม: ประตู D1 ผนังแนวกริด 1 และ 11 (A101) ระดับต่างกัน 0.50 ม.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="37" t="inlineStr">
         <is>
-          <t>4.1.4</t>
+          <t>4.1.1</t>
         </is>
       </c>
       <c r="B75" s="39" t="inlineStr">
@@ -8512,63 +8644,63 @@
       </c>
       <c r="C75" s="37" t="inlineStr">
         <is>
-          <t>พื้น AF01 / SF02 ระดับถนน</t>
+          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับพื้นถนนรอบอาคาร (I22-22) รวมค่าตอก</t>
         </is>
       </c>
       <c r="D75" s="37" t="inlineStr">
         <is>
-          <t>AF01 16.88 + SF02 93.26 ตร.ม. คอนกรีต 25.76 ลบ.ม. (S6.1)</t>
+          <t>กลุ่มเข็มถนน: ผู้ว่าจ้างยืนยัน 249 ต้น (ผัง S201/S202 แสดงตำแหน่ง 232 ต้น ขอตำแหน่งอีก 17 ต้นจากผู้ออกแบบ)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="37" t="inlineStr">
         <is>
-          <t>4.1.5</t>
-        </is>
-      </c>
-      <c r="B76" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.1.2</t>
+        </is>
+      </c>
+      <c r="B76" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C76" s="37" t="inlineStr">
         <is>
-          <t>ทราย/หินคลุกรองใต้พื้นถนน S2 หนา 0.10 ม. บดอัด</t>
+          <t>ฐาน F1A 0.60x0.60x0.30 ม. รับพื้นถนน</t>
         </is>
       </c>
       <c r="D76" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: 2,440.69 ตร.ม. x 0.10 ม. (ความหนาสมมติ รอแบบ)</t>
+          <t>ตามเข็มถนน 249 ต้น คอนกรีต 26.78, ทราย 35.86, คอนกรีตหยาบ 6.10 ลบ.ม. (S1.1)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="37" t="inlineStr">
         <is>
-          <t>4.1.6</t>
-        </is>
-      </c>
-      <c r="B77" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.1.3</t>
+        </is>
+      </c>
+      <c r="B77" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C77" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม/ตะแกรงเหล็ก พื้นถนน และฐาน F1A</t>
+          <t>พื้นถนน S2 คสล. หนา 0.15 ม. TOP ±0.00 พร้อมรอยต่อ/ตัดรอยต่อ</t>
         </is>
       </c>
       <c r="D77" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม</t>
+          <t>คอนกรีต 366.10 ลบ.ม. (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="37" t="inlineStr">
         <is>
-          <t>4.2.1</t>
+          <t>4.1.4</t>
         </is>
       </c>
       <c r="B78" s="39" t="inlineStr">
@@ -8578,19 +8710,19 @@
       </c>
       <c r="C78" s="37" t="inlineStr">
         <is>
-          <t>ทางลาดขนส่ง คสล. กว้าง 6.00 ม. (ด้านเหนือแนวกริด 5-6 และด้านใต้แนวกริด 7-8)</t>
+          <t>พื้น AF01 / SF02 ระดับถนน</t>
         </is>
       </c>
       <c r="D78" s="37" t="inlineStr">
         <is>
-          <t>A101/S202 ขนาดวัดจากผัง</t>
+          <t>AF01 16.88 + SF02 93.26 ตร.ม. คอนกรีต 25.76 ลบ.ม. (S6.1)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="37" t="inlineStr">
         <is>
-          <t>4.3.1</t>
+          <t>4.1.5</t>
         </is>
       </c>
       <c r="B79" s="40" t="inlineStr">
@@ -8600,41 +8732,41 @@
       </c>
       <c r="C79" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
+          <t>ทราย/หินคลุกรองใต้พื้นถนน S2 หนา 0.10 ม. บดอัด</t>
         </is>
       </c>
       <c r="D79" s="37" t="inlineStr">
         <is>
-          <t>S2 / S201 = 6 ต้น; A104 แสดง 3x3 = 9 ต้น (ยืนยัน)</t>
+          <t>เพิ่ม: 2,440.69 ตร.ม. x 0.10 ม. (ความหนาสมมติ รอแบบ)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="37" t="inlineStr">
         <is>
-          <t>4.3.2</t>
-        </is>
-      </c>
-      <c r="B80" s="38" t="inlineStr">
-        <is>
-          <t>แก้ไข</t>
+          <t>4.1.6</t>
+        </is>
+      </c>
+      <c r="B80" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C80" s="37" t="inlineStr">
         <is>
-          <t>แท่นหม้อแปลง 750 kVA คสล.: ฐาน 5.00x3.00x0.40 ม. + แท่น 3.50x1.75x0.15 ม. (A104)</t>
+          <t>เหล็กเสริม/ตะแกรงเหล็ก พื้นถนน และฐาน F1A</t>
         </is>
       </c>
       <c r="D80" s="37" t="inlineStr">
         <is>
-          <t>แบบ A104: คอนกรีต 6.00 + 0.92 ลบ.ม. ไม้แบบ 7.98 ตร.ม.; A104 แสดงเข็ม 9 ต้น แต่ S201 แสดง 6 ต้น (ยืนยัน)</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="37" t="inlineStr">
         <is>
-          <t>4.4.1</t>
+          <t>4.2.1</t>
         </is>
       </c>
       <c r="B81" s="39" t="inlineStr">
@@ -8644,107 +8776,107 @@
       </c>
       <c r="C81" s="37" t="inlineStr">
         <is>
-          <t>ขุดดินถังเก็บน้ำใต้ดิน ~12.12 x 6.63 ม. ลึก 3.00 ม. และขนทิ้ง</t>
+          <t>ทางลาดขนส่ง คสล. กว้าง 6.00 ม. (ด้านเหนือแนวกริด 5-6 และด้านใต้แนวกริด 7-8)</t>
         </is>
       </c>
       <c r="D81" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ขนาดจากเวกเตอร์ S201/S202 ลึกจาก ±0.00 ถึงใต้คอนกรีตหยาบ -3.00</t>
+          <t>A101/S202 ขนาดวัดจากผัง</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="37" t="inlineStr">
         <is>
-          <t>4.4.2</t>
-        </is>
-      </c>
-      <c r="B82" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>4.3.1</t>
+        </is>
+      </c>
+      <c r="B82" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C82" s="37" t="inlineStr">
         <is>
-          <t>พื้นถังเก็บน้ำใต้ดิน คสล. หนา 0.25 ม. (TF -2.60 / BF -2.85) พร้อมคอนกรีตหยาบ/ทราย</t>
+          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
         </is>
       </c>
       <c r="D82" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: 12.12 x 6.63 ม. คอนกรีต 20.09 ลบ.ม. (S202)</t>
+          <t>S2 / S201 = 6 ต้น; A104 แสดง 3x3 = 9 ต้น (ยืนยัน)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="37" t="inlineStr">
         <is>
-          <t>4.4.3</t>
-        </is>
-      </c>
-      <c r="B83" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.3.2</t>
+        </is>
+      </c>
+      <c r="B83" s="38" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
         </is>
       </c>
       <c r="C83" s="37" t="inlineStr">
         <is>
-          <t>ผนัง ฝา ช่องเปิด บ่อพัก บันไดลิง และกันซึม ถังเก็บน้ำใต้ดิน</t>
+          <t>แท่นหม้อแปลง 750 kVA คสล.: ฐาน 5.00x3.00x0.40 ม. + แท่น 3.50x1.75x0.15 ม. (A104)</t>
         </is>
       </c>
       <c r="D83" s="37" t="inlineStr">
         <is>
-          <t>รอแบบขยาย (S202 แสดงเฉพาะพื้นถัง)</t>
+          <t>แบบ A104: คอนกรีต 6.00 + 0.92 ลบ.ม. ไม้แบบ 7.98 ตร.ม.; A104 แสดงเข็ม 9 ต้น แต่ S201 แสดง 6 ต้น (ยืนยัน)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="37" t="inlineStr">
         <is>
-          <t>4.4.4</t>
-        </is>
-      </c>
-      <c r="B84" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.4.1</t>
+        </is>
+      </c>
+      <c r="B84" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C84" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริมถังเก็บน้ำใต้ดิน</t>
+          <t>ขุดดินถังเก็บน้ำใต้ดิน ~12.12 x 6.63 ม. ลึก 3.00 ม. และขนทิ้ง</t>
         </is>
       </c>
       <c r="D84" s="37" t="inlineStr">
         <is>
-          <t>รอเอกสารออกแบบเหล็กเสริม</t>
+          <t>เพิ่ม: ขนาดจากเวกเตอร์ S201/S202 ลึกจาก ±0.00 ถึงใต้คอนกรีตหยาบ -3.00</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="37" t="inlineStr">
         <is>
-          <t>4.5.1</t>
-        </is>
-      </c>
-      <c r="B85" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.4.2</t>
+        </is>
+      </c>
+      <c r="B85" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C85" s="37" t="inlineStr">
         <is>
-          <t>รางระบายน้ำ คสล. พร้อมฝาปิด ตามแนวเขตที่ดิน</t>
+          <t>พื้นถังเก็บน้ำใต้ดิน คสล. หนา 0.25 ม. (TF -2.60 / BF -2.85) พร้อมคอนกรีตหยาบ/ทราย</t>
         </is>
       </c>
       <c r="D85" s="37" t="inlineStr">
         <is>
-          <t>A101 ขนาดรางรอแบบขยาย</t>
+          <t>เพิ่ม: 12.12 x 6.63 ม. คอนกรีต 20.09 ลบ.ม. (S202)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="37" t="inlineStr">
         <is>
-          <t>4.5.2</t>
+          <t>4.4.3</t>
         </is>
       </c>
       <c r="B86" s="40" t="inlineStr">
@@ -8754,41 +8886,41 @@
       </c>
       <c r="C86" s="37" t="inlineStr">
         <is>
-          <t>บ่อพัก/บ่อบำบัด และจุดเชื่อมท่อระบายสาธารณะ</t>
+          <t>ผนัง ฝา ช่องเปิด บ่อพัก บันไดลิง และกันซึม ถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="D86" s="37" t="inlineStr">
         <is>
-          <t>รอแบบ</t>
+          <t>รอแบบขยาย (S202 แสดงเฉพาะพื้นถัง)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="37" t="inlineStr">
         <is>
-          <t>4.5.3</t>
-        </is>
-      </c>
-      <c r="B87" s="39" t="inlineStr">
-        <is>
-          <t>เพิ่มใหม่</t>
+          <t>4.4.4</t>
+        </is>
+      </c>
+      <c r="B87" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
         </is>
       </c>
       <c r="C87" s="37" t="inlineStr">
         <is>
-          <t>ท่อระบายน้ำฝนใต้ดิน PVC Ø4" จากท่อลงถึงรางระบายน้ำ</t>
+          <t>เหล็กเสริมถังเก็บน้ำใต้ดิน</t>
         </is>
       </c>
       <c r="D87" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: ท่อลง 10 จุด (3.1.5)</t>
+          <t>รอเอกสารออกแบบเหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="37" t="inlineStr">
         <is>
-          <t>4.6.1</t>
+          <t>4.5.1</t>
         </is>
       </c>
       <c r="B88" s="40" t="inlineStr">
@@ -8798,19 +8930,19 @@
       </c>
       <c r="C88" s="37" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-260x260 + ฐาน 0.66x0.66 ม. แนวเขตที่ดินด้านใต้และตะวันออก (ไม่มีใน BOQ/ตาราง S2)</t>
+          <t>รางระบายน้ำ คสล. พร้อมฝาปิด ตามแนวเขตที่ดิน</t>
         </is>
       </c>
       <c r="D88" s="37" t="inlineStr">
         <is>
-          <t>พบในผัง S201 16 จุด ยังไม่ทราบหน้าที่ (เสารั้ว/เสาไฟ/ป้าย?) สอบถามผู้ออกแบบ</t>
+          <t>A101 ขนาดรางรอแบบขยาย</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="37" t="inlineStr">
         <is>
-          <t>4.6.2</t>
+          <t>4.5.2</t>
         </is>
       </c>
       <c r="B89" s="40" t="inlineStr">
@@ -8820,41 +8952,41 @@
       </c>
       <c r="C89" s="37" t="inlineStr">
         <is>
-          <t>รั้วถาวร / ประตูทางเข้าโครงการ</t>
+          <t>บ่อพัก/บ่อบำบัด และจุดเชื่อมท่อระบายสาธารณะ</t>
         </is>
       </c>
       <c r="D89" s="37" t="inlineStr">
         <is>
-          <t>ไม่มีในแบบ ยืนยันว่าอยู่ในขอบเขตหรือไม่</t>
+          <t>รอแบบ</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="37" t="inlineStr">
         <is>
-          <t>5.1.1</t>
-        </is>
-      </c>
-      <c r="B90" s="40" t="inlineStr">
-        <is>
-          <t>รอข้อมูล</t>
+          <t>4.5.3</t>
+        </is>
+      </c>
+      <c r="B90" s="39" t="inlineStr">
+        <is>
+          <t>เพิ่มใหม่</t>
         </is>
       </c>
       <c r="C90" s="37" t="inlineStr">
         <is>
-          <t>ระบบไฟฟ้าแสงสว่างและเต้ารับภายในอาคารโกดัง 3,240 ตร.ม. และไฟส่องสว่างภายนอก</t>
+          <t>ท่อระบายน้ำฝนใต้ดิน PVC Ø4" จากท่อลงถึงรางระบายน้ำ</t>
         </is>
       </c>
       <c r="D90" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum</t>
+          <t>เพิ่ม: ท่อลง 10 จุด (3.1.5)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="37" t="inlineStr">
         <is>
-          <t>5.1.2</t>
+          <t>4.6.1</t>
         </is>
       </c>
       <c r="B91" s="40" t="inlineStr">
@@ -8864,19 +8996,19 @@
       </c>
       <c r="C91" s="37" t="inlineStr">
         <is>
-          <t>สายเมนและท่อร้อยสายใต้ดินจากหม้อแปลงถึงห้อง MDB</t>
+          <t>เสาเข็ม I-260x260 + ฐาน 0.66x0.66 ม. แนวเขตที่ดินด้านใต้และตะวันออก (ไม่มีใน BOQ/ตาราง S2)</t>
         </is>
       </c>
       <c r="D91" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum (ระยะประมาณ 10 ม.)</t>
+          <t>พบในผัง S201 16 จุด ยังไม่ทราบหน้าที่ (เสารั้ว/เสาไฟ/ป้าย?) สอบถามผู้ออกแบบ</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="37" t="inlineStr">
         <is>
-          <t>5.1.3</t>
+          <t>4.6.2</t>
         </is>
       </c>
       <c r="B92" s="40" t="inlineStr">
@@ -8886,19 +9018,19 @@
       </c>
       <c r="C92" s="37" t="inlineStr">
         <is>
-          <t>ระบบป้องกันฟ้าผ่าและสายดิน อาคารสูง +15.25 ม.</t>
+          <t>รั้วถาวร / ประตูทางเข้าโครงการ</t>
         </is>
       </c>
       <c r="D92" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum</t>
+          <t>ไม่มีในแบบ ยืนยันว่าอยู่ในขอบเขตหรือไม่</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="37" t="inlineStr">
         <is>
-          <t>5.1.4</t>
+          <t>5.1.1</t>
         </is>
       </c>
       <c r="B93" s="40" t="inlineStr">
@@ -8908,7 +9040,7 @@
       </c>
       <c r="C93" s="37" t="inlineStr">
         <is>
-          <t>ระบบสุขาภิบาลและถังบำบัดน้ำเสียสำเร็จรูป อาคารห้องน้ำ</t>
+          <t>ระบบไฟฟ้าแสงสว่างและเต้ารับภายในอาคารโกดัง 3,240 ตร.ม. และไฟส่องสว่างภายนอก</t>
         </is>
       </c>
       <c r="D93" s="37" t="inlineStr">
@@ -8920,7 +9052,7 @@
     <row r="94">
       <c r="A94" s="37" t="inlineStr">
         <is>
-          <t>5.1.5</t>
+          <t>5.1.2</t>
         </is>
       </c>
       <c r="B94" s="40" t="inlineStr">
@@ -8930,105 +9062,129 @@
       </c>
       <c r="C94" s="37" t="inlineStr">
         <is>
-          <t>ระบบน้ำประปา ปั๊มน้ำ และท่อจากถังเก็บน้ำใต้ดิน</t>
+          <t>สายเมนและท่อร้อยสายใต้ดินจากหม้อแปลงถึงห้อง MDB</t>
         </is>
       </c>
       <c r="D94" s="37" t="inlineStr">
         <is>
-          <t>เพิ่ม: Provisional sum</t>
+          <t>เพิ่ม: Provisional sum (ระยะประมาณ 10 ม.)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="37" t="inlineStr">
         <is>
+          <t>5.1.3</t>
+        </is>
+      </c>
+      <c r="B95" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
+        </is>
+      </c>
+      <c r="C95" s="37" t="inlineStr">
+        <is>
+          <t>ระบบป้องกันฟ้าผ่าและสายดิน อาคารสูง +15.25 ม.</t>
+        </is>
+      </c>
+      <c r="D95" s="37" t="inlineStr">
+        <is>
+          <t>เพิ่ม: Provisional sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="37" t="inlineStr">
+        <is>
+          <t>5.1.4</t>
+        </is>
+      </c>
+      <c r="B96" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
+        </is>
+      </c>
+      <c r="C96" s="37" t="inlineStr">
+        <is>
+          <t>ระบบสุขาภิบาลและถังบำบัดน้ำเสียสำเร็จรูป อาคารห้องน้ำ</t>
+        </is>
+      </c>
+      <c r="D96" s="37" t="inlineStr">
+        <is>
+          <t>เพิ่ม: Provisional sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="37" t="inlineStr">
+        <is>
+          <t>5.1.5</t>
+        </is>
+      </c>
+      <c r="B97" s="40" t="inlineStr">
+        <is>
+          <t>รอข้อมูล</t>
+        </is>
+      </c>
+      <c r="C97" s="37" t="inlineStr">
+        <is>
+          <t>ระบบน้ำประปา ปั๊มน้ำ และท่อจากถังเก็บน้ำใต้ดิน</t>
+        </is>
+      </c>
+      <c r="D97" s="37" t="inlineStr">
+        <is>
+          <t>เพิ่ม: Provisional sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="37" t="inlineStr">
+        <is>
           <t>5.1.6</t>
         </is>
       </c>
-      <c r="B95" s="40" t="inlineStr">
+      <c r="B98" s="40" t="inlineStr">
         <is>
           <t>รอข้อมูล</t>
         </is>
       </c>
-      <c r="C95" s="37" t="inlineStr">
+      <c r="C98" s="37" t="inlineStr">
         <is>
           <t>อุปกรณ์ดับเพลิง ป้ายทางออก ไฟฉุกเฉิน และระบบแจ้งเหตุเพลิงไหม้</t>
         </is>
       </c>
-      <c r="D95" s="37" t="inlineStr">
+      <c r="D98" s="37" t="inlineStr">
         <is>
           <t>เพิ่ม: Provisional sum</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="37" t="n"/>
-      <c r="B96" s="37" t="n"/>
-      <c r="C96" s="37" t="n"/>
-      <c r="D96" s="37" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="37" t="inlineStr"/>
-      <c r="B97" s="41" t="inlineStr">
-        <is>
-          <t>ข้อสังเกต</t>
-        </is>
-      </c>
-      <c r="C97" s="37" t="inlineStr"/>
-      <c r="D97" s="37" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="37" t="inlineStr"/>
-      <c r="B98" s="37" t="inlineStr">
-        <is>
-          <t>ขอบเขต</t>
-        </is>
-      </c>
-      <c r="C98" s="37" t="inlineStr">
-        <is>
-          <t>งานระบบไฟฟ้า ประปา สุขาภิบาล ดับเพลิง (MEP) ไม่มีแบบ เสนอเป็นเงินสำรองในหมวด 5 ให้ผู้ว่าจ้างยืนยันขอบเขตก่อนสรุปราคา</t>
-        </is>
-      </c>
-      <c r="D98" s="37" t="inlineStr"/>
-    </row>
     <row r="99">
-      <c r="A99" s="37" t="inlineStr"/>
-      <c r="B99" s="37" t="inlineStr">
-        <is>
-          <t>แบบ</t>
-        </is>
-      </c>
-      <c r="C99" s="37" t="inlineStr">
-        <is>
-          <t>กรอบชื่อแบบทุกแผ่นระบุ 'แบบก่อสร้างบ้านพักอาศัย คสล 1 ชั้น' และ Date 03/31/22 ควรแก้ก่อนแนบประกอบใบเสนอราคา</t>
-        </is>
-      </c>
-      <c r="D99" s="37" t="inlineStr"/>
+      <c r="A99" s="37" t="n"/>
+      <c r="B99" s="37" t="n"/>
+      <c r="C99" s="37" t="n"/>
+      <c r="D99" s="37" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="37" t="inlineStr"/>
-      <c r="B100" s="37" t="inlineStr">
-        <is>
-          <t>แบบ</t>
-        </is>
-      </c>
-      <c r="C100" s="37" t="inlineStr">
-        <is>
-          <t>แบบไม่มีลูกศรทิศเหนือ ผู้ว่าจ้างยืนยันให้ด้านแนวกริด A เป็นทิศเหนือสำหรับทำแบบ</t>
-        </is>
-      </c>
+      <c r="B100" s="41" t="inlineStr">
+        <is>
+          <t>ข้อสังเกต</t>
+        </is>
+      </c>
+      <c r="C100" s="37" t="inlineStr"/>
       <c r="D100" s="37" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="37" t="inlineStr"/>
       <c r="B101" s="37" t="inlineStr">
         <is>
-          <t>แบบ</t>
+          <t>ขอบเขต</t>
         </is>
       </c>
       <c r="C101" s="37" t="inlineStr">
         <is>
-          <t>ตาราง S2 นับเข็ม 737 ต้น แต่ผัง S201 นับได้ 734 ต้น (+16 ต้นใต้ฐาน 0.66 ม. ที่ไม่อยู่ในตาราง) และ F2P ผู้ว่าจ้างยืนยัน 46 ฐาน (ตาราง S1.1 นับ 47 ผิด เสาเหล็ก H250x175 จึงเป็น 46 ต้น)</t>
+          <t>งานระบบไฟฟ้า ประปา สุขาภิบาล ดับเพลิง (MEP) ไม่มีแบบ เสนอเป็นเงินสำรองในหมวด 5 ให้ผู้ว่าจ้างยืนยันขอบเขตก่อนสรุปราคา</t>
         </is>
       </c>
       <c r="D101" s="37" t="inlineStr"/>
@@ -9037,12 +9193,12 @@
       <c r="A102" s="37" t="inlineStr"/>
       <c r="B102" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม</t>
+          <t>แบบ</t>
         </is>
       </c>
       <c r="C102" s="37" t="inlineStr">
         <is>
-          <t>เหล็กเสริม คสล. ทุกรายการรอเอกสารการออกแบบเหล็กเสริมจากผู้ออกแบบ ตัวเลขในหมายเหตุเป็นค่าอ้างอิงเท่านั้น ไม่ใช้เป็นปริมาณ</t>
+          <t>กรอบชื่อแบบทุกแผ่นระบุ 'แบบก่อสร้างบ้านพักอาศัย คสล 1 ชั้น' และ Date 03/31/22 ควรแก้ก่อนแนบประกอบใบเสนอราคา</t>
         </is>
       </c>
       <c r="D102" s="37" t="inlineStr"/>
@@ -9051,12 +9207,12 @@
       <c r="A103" s="37" t="inlineStr"/>
       <c r="B103" s="37" t="inlineStr">
         <is>
-          <t>โครงหลังคา</t>
+          <t>แบบ</t>
         </is>
       </c>
       <c r="C103" s="37" t="inlineStr">
         <is>
-          <t>ยังไม่มีแบบโครงสร้างหลังคา น้ำหนักเหล็กโครงถัก/แป/ค้ำยันเป็นค่าประมาณจากโมเดล BIM</t>
+          <t>แบบไม่มีลูกศรทิศเหนือ ผู้ว่าจ้างยืนยันให้ด้านแนวกริด A เป็นทิศเหนือสำหรับทำแบบ</t>
         </is>
       </c>
       <c r="D103" s="37" t="inlineStr"/>
@@ -9065,15 +9221,57 @@
       <c r="A104" s="37" t="inlineStr"/>
       <c r="B104" s="37" t="inlineStr">
         <is>
+          <t>แบบ</t>
+        </is>
+      </c>
+      <c r="C104" s="37" t="inlineStr">
+        <is>
+          <t>ตาราง S2 นับเข็ม 737 ต้น แต่ผัง S201 นับได้ 734 ต้น (+16 ต้นใต้ฐาน 0.66 ม. ที่ไม่อยู่ในตาราง) และ F2P ผู้ว่าจ้างยืนยัน 46 ฐาน (ตาราง S1.1 นับ 47 ผิด เสาเหล็ก H250x175 จึงเป็น 46 ต้น)</t>
+        </is>
+      </c>
+      <c r="D104" s="37" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="37" t="inlineStr"/>
+      <c r="B105" s="37" t="inlineStr">
+        <is>
+          <t>เหล็กเสริม</t>
+        </is>
+      </c>
+      <c r="C105" s="37" t="inlineStr">
+        <is>
+          <t>เหล็กเสริม คสล. ทุกรายการรอเอกสารการออกแบบเหล็กเสริมจากผู้ออกแบบ ตัวเลขในหมายเหตุเป็นค่าอ้างอิงเท่านั้น ไม่ใช้เป็นปริมาณ</t>
+        </is>
+      </c>
+      <c r="D105" s="37" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="37" t="inlineStr"/>
+      <c r="B106" s="37" t="inlineStr">
+        <is>
+          <t>โครงหลังคา</t>
+        </is>
+      </c>
+      <c r="C106" s="37" t="inlineStr">
+        <is>
+          <t>ยังไม่มีแบบโครงสร้างหลังคา น้ำหนักเหล็กโครงถัก/แป/ค้ำยันเป็นค่าประมาณจากโมเดล BIM</t>
+        </is>
+      </c>
+      <c r="D106" s="37" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="37" t="inlineStr"/>
+      <c r="B107" s="37" t="inlineStr">
+        <is>
           <t>ดินถม</t>
         </is>
       </c>
-      <c r="C104" s="37" t="inlineStr">
+      <c r="C107" s="37" t="inlineStr">
         <is>
           <t>ผู้ว่าจ้างยืนยัน 27/10/69: ดินเดิมอยู่ที่ ±0.00 (ระดับถนนรอบอาคาร) ระดับ -1.50 คือถนนสาธารณะ คิด BOQ ถมหนา 0.30 ม. ปริมาณจริงเบิกตามผลสำรวจระดับ P1.2</t>
         </is>
       </c>
-      <c r="D104" s="37" t="inlineStr"/>
+      <c r="D107" s="37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9473,7 +9671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10371,11 +10569,11 @@
       </c>
       <c r="B26" s="46" t="inlineStr">
         <is>
-          <t>เสาเหล็ก H250x175x44.1 กก./ม. บนหัวเสา คสล. +4.50 ถึง +9.00 พร้อมแผ่นเหล็กฐาน Anchor bolt</t>
+          <t>เสาเหล็ก H244x175x7x11 (H250x175) 44.1 กก./ม. จากแผ่นเหล็กฐาน +4.545 ถึงใต้แผ่นหัวเสา +8.98</t>
         </is>
       </c>
       <c r="C26" s="46" t="n">
-        <v>9311</v>
+        <v>8997</v>
       </c>
       <c r="D26" s="46" t="inlineStr">
         <is>
@@ -10383,7 +10581,7 @@
         </is>
       </c>
       <c r="E26" s="46" t="n">
-        <v>9310.84</v>
+        <v>8996.84</v>
       </c>
       <c r="F26" s="46" t="n">
         <v>0</v>
@@ -10395,7 +10593,7 @@
       </c>
       <c r="H26" s="46" t="inlineStr">
         <is>
-          <t>เสา 46 ต้น (ผัง S201) x 4.59 ม. x 44.1 กก./ม.</t>
+          <t>โมเดล เสาเหล็ก 46 ต้น</t>
         </is>
       </c>
     </row>
@@ -10483,7 +10681,7 @@
         </is>
       </c>
       <c r="C29" s="46" t="n">
-        <v>5880</v>
+        <v>5849</v>
       </c>
       <c r="D29" s="46" t="inlineStr">
         <is>
@@ -10491,7 +10689,7 @@
         </is>
       </c>
       <c r="E29" s="46" t="n">
-        <v>5879.97</v>
+        <v>5848.55</v>
       </c>
       <c r="F29" s="46" t="n">
         <v>0</v>
@@ -10515,7 +10713,7 @@
       </c>
       <c r="B30" s="46" t="inlineStr">
         <is>
-          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) ใต้แผ่นฐานเสาเหล็ก</t>
+          <t>ปูนเกราท์ไม่หดตัว (Non-shrink grout) หนา 25 มม. ใต้แผ่นเหล็กฐาน</t>
         </is>
       </c>
       <c r="C30" s="46" t="n">
@@ -10546,16 +10744,16 @@
     <row r="31">
       <c r="A31" s="46" t="inlineStr">
         <is>
-          <t>2.6.1</t>
+          <t>2.5.7</t>
         </is>
       </c>
       <c r="B31" s="46" t="inlineStr">
         <is>
-          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
+          <t>แผ่นเหล็กฐาน (Base plate) PL 20x200x450 มม. เจาะรู 6 รู เชื่อมกับเสาเหล็ก</t>
         </is>
       </c>
       <c r="C31" s="46" t="n">
-        <v>6703</v>
+        <v>649.98</v>
       </c>
       <c r="D31" s="46" t="inlineStr">
         <is>
@@ -10563,10 +10761,10 @@
         </is>
       </c>
       <c r="E31" s="46" t="n">
-        <v>6703.2</v>
+        <v>649.98</v>
       </c>
       <c r="F31" s="46" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G31" s="47" t="inlineStr">
         <is>
@@ -10575,23 +10773,23 @@
       </c>
       <c r="H31" s="46" t="inlineStr">
         <is>
-          <t>ตาราง S4.1 100.80 ม. x 66.5 กก./ม.</t>
+          <t>โมเดล แผ่นเหล็กฐาน</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="46" t="inlineStr">
         <is>
-          <t>2.6.2</t>
+          <t>2.5.8</t>
         </is>
       </c>
       <c r="B32" s="46" t="inlineStr">
         <is>
-          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
+          <t>แผ่นเหล็กหัวเสา (Top plate) PL 20x200x450 มม. ที่ +9.00 รับโครงถัก</t>
         </is>
       </c>
       <c r="C32" s="46" t="n">
-        <v>5219</v>
+        <v>649.98</v>
       </c>
       <c r="D32" s="46" t="inlineStr">
         <is>
@@ -10599,7 +10797,7 @@
         </is>
       </c>
       <c r="E32" s="46" t="n">
-        <v>5218.5</v>
+        <v>649.98</v>
       </c>
       <c r="F32" s="46" t="n">
         <v>0</v>
@@ -10611,31 +10809,31 @@
       </c>
       <c r="H32" s="46" t="inlineStr">
         <is>
-          <t>โมเดล</t>
+          <t>โมเดล แผ่นหัวเสา</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="46" t="inlineStr">
         <is>
-          <t>2.6.3</t>
+          <t>2.5.9</t>
         </is>
       </c>
       <c r="B33" s="46" t="inlineStr">
         <is>
-          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
+          <t>Anchor bolt M20 ยาว 750 มม. ปลายงอ พร้อมแป้นเกลียว 2 ตัว แหวน และแบบจับตำแหน่ง (Template) ฝังในหัวเสา คสล.</t>
         </is>
       </c>
       <c r="C33" s="46" t="n">
-        <v>306.15</v>
+        <v>276</v>
       </c>
       <c r="D33" s="46" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
+          <t>ชุด</t>
         </is>
       </c>
       <c r="E33" s="46" t="n">
-        <v>306.15</v>
+        <v>276</v>
       </c>
       <c r="F33" s="46" t="n">
         <v>0</v>
@@ -10647,34 +10845,34 @@
       </c>
       <c r="H33" s="46" t="inlineStr">
         <is>
-          <t>ตาราง S6.1</t>
+          <t>โมเดล Anchor bolt</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="46" t="inlineStr">
         <is>
-          <t>2.6.5</t>
+          <t>2.6.1</t>
         </is>
       </c>
       <c r="B34" s="46" t="inlineStr">
         <is>
-          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
+          <t>เสาเหล็กชั้นลอย H250x250x66.5 กก./ม.</t>
         </is>
       </c>
       <c r="C34" s="46" t="n">
-        <v>33.6</v>
+        <v>6703</v>
       </c>
       <c r="D34" s="46" t="inlineStr">
         <is>
-          <t>ม.</t>
+          <t>กก.</t>
         </is>
       </c>
       <c r="E34" s="46" t="n">
-        <v>33.6</v>
+        <v>6703.2</v>
       </c>
       <c r="F34" s="46" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G34" s="47" t="inlineStr">
         <is>
@@ -10683,34 +10881,34 @@
       </c>
       <c r="H34" s="46" t="inlineStr">
         <is>
-          <t>โมเดลชั้นลอย</t>
+          <t>ตาราง S4.1 100.80 ม. x 66.5 กก./ม.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="46" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>2.6.2</t>
         </is>
       </c>
       <c r="B35" s="46" t="inlineStr">
         <is>
-          <t>หลังคาเมทัลชีทหนา 0.47 มม. พร้อมฉนวน PU 25 มม. (พื้นที่ตามลาด)</t>
+          <t>คานเหล็กชั้นลอย (หน้าตัดรอแบบ)</t>
         </is>
       </c>
       <c r="C35" s="46" t="n">
-        <v>3395</v>
+        <v>5219</v>
       </c>
       <c r="D35" s="46" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
+          <t>กก.</t>
         </is>
       </c>
       <c r="E35" s="46" t="n">
-        <v>3395.07</v>
+        <v>5218.5</v>
       </c>
       <c r="F35" s="46" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G35" s="47" t="inlineStr">
         <is>
@@ -10726,16 +10924,16 @@
     <row r="36">
       <c r="A36" s="46" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>2.6.3</t>
         </is>
       </c>
       <c r="B36" s="46" t="inlineStr">
         <is>
-          <t>Jack roof กว้าง 6.00 ม. ยาว 42.00 ม. สัน +15.25 พร้อมตะแกรงระบายอากาศ</t>
+          <t>พื้นชั้นลอย F8 (Metal deck/พื้นสำเร็จ ตามแบบ)</t>
         </is>
       </c>
       <c r="C36" s="46" t="n">
-        <v>252</v>
+        <v>306.15</v>
       </c>
       <c r="D36" s="46" t="inlineStr">
         <is>
@@ -10743,7 +10941,7 @@
         </is>
       </c>
       <c r="E36" s="46" t="n">
-        <v>252</v>
+        <v>306.15</v>
       </c>
       <c r="F36" s="46" t="n">
         <v>0</v>
@@ -10755,23 +10953,23 @@
       </c>
       <c r="H36" s="46" t="inlineStr">
         <is>
-          <t>A202 / โมเดล</t>
+          <t>ตาราง S6.1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="46" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>2.6.5</t>
         </is>
       </c>
       <c r="B37" s="46" t="inlineStr">
         <is>
-          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30 ม.</t>
+          <t>ราวกันตกเหล็กขอบชั้นลอยด้านเปิด สูง 1.10 ม.</t>
         </is>
       </c>
       <c r="C37" s="46" t="n">
-        <v>110</v>
+        <v>33.6</v>
       </c>
       <c r="D37" s="46" t="inlineStr">
         <is>
@@ -10779,7 +10977,7 @@
         </is>
       </c>
       <c r="E37" s="46" t="n">
-        <v>110</v>
+        <v>33.6</v>
       </c>
       <c r="F37" s="46" t="n">
         <v>0</v>
@@ -10791,23 +10989,23 @@
       </c>
       <c r="H37" s="46" t="inlineStr">
         <is>
-          <t>โมเดล</t>
+          <t>โมเดลชั้นลอย</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="46" t="inlineStr">
         <is>
-          <t>3.1.6</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="B38" s="46" t="inlineStr">
         <is>
-          <t>ผนังเมทัลชีท ระดับ +5.20 ถึงชายคา/จั่ว</t>
+          <t>หลังคาเมทัลชีทหนา 0.47 มม. พร้อมฉนวน PU 25 มม. (พื้นที่ตามลาด)</t>
         </is>
       </c>
       <c r="C38" s="46" t="n">
-        <v>1379</v>
+        <v>3395</v>
       </c>
       <c r="D38" s="46" t="inlineStr">
         <is>
@@ -10815,10 +11013,10 @@
         </is>
       </c>
       <c r="E38" s="46" t="n">
-        <v>1379</v>
+        <v>3395.07</v>
       </c>
       <c r="F38" s="46" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G38" s="47" t="inlineStr">
         <is>
@@ -10834,24 +11032,24 @@
     <row r="39">
       <c r="A39" s="46" t="inlineStr">
         <is>
-          <t>3.1.7</t>
+          <t>3.1.2</t>
         </is>
       </c>
       <c r="B39" s="46" t="inlineStr">
         <is>
-          <t>ตะแกรงกันนก/ช่องระบายอากาศ ระดับ +4.50 ถึง +5.20 รอบอาคาร</t>
+          <t>Jack roof กว้าง 6.00 ม. ยาว 42.00 ม. สัน +15.25 พร้อมตะแกรงระบายอากาศ</t>
         </is>
       </c>
       <c r="C39" s="46" t="n">
-        <v>216</v>
+        <v>252</v>
       </c>
       <c r="D39" s="46" t="inlineStr">
         <is>
-          <t>ม.</t>
+          <t>ตร.ม.</t>
         </is>
       </c>
       <c r="E39" s="46" t="n">
-        <v>216</v>
+        <v>252</v>
       </c>
       <c r="F39" s="46" t="n">
         <v>0</v>
@@ -10863,34 +11061,34 @@
       </c>
       <c r="H39" s="46" t="inlineStr">
         <is>
-          <t>เส้นรอบอาคาร - ประตูม้วน</t>
+          <t>A202 / โมเดล</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="46" t="inlineStr">
         <is>
-          <t>3.2.1</t>
+          <t>3.1.4</t>
         </is>
       </c>
       <c r="B40" s="46" t="inlineStr">
         <is>
-          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ม. +0.50 ถึง +4.35 (ต่ำกว่าหัวเสา คสล. 0.15 ม.)</t>
+          <t>รางน้ำฝนเหล็กอาบสังกะสี 0.30x0.30 ม.</t>
         </is>
       </c>
       <c r="C40" s="46" t="n">
-        <v>750.67</v>
+        <v>110</v>
       </c>
       <c r="D40" s="46" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
+          <t>ม.</t>
         </is>
       </c>
       <c r="E40" s="46" t="n">
-        <v>744.63</v>
+        <v>110</v>
       </c>
       <c r="F40" s="46" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="G40" s="47" t="inlineStr">
         <is>
@@ -10899,34 +11097,34 @@
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
-          <t>โมเดล (ผนัง W1 หักเสาเอ็น/คานเอ็น/ประตู)</t>
+          <t>โมเดล</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="46" t="inlineStr">
         <is>
-          <t>3.2.3</t>
+          <t>3.1.6</t>
         </is>
       </c>
       <c r="B41" s="46" t="inlineStr">
         <is>
-          <t>คานทับหลัง คสล. 0.15x0.15 ม. ระดับ +4.35 ถึง +4.50 (คอนกรีต ไม้แบบ)</t>
+          <t>ผนังเมทัลชีท ระดับ +5.20 ถึงชายคา/จั่ว</t>
         </is>
       </c>
       <c r="C41" s="46" t="n">
-        <v>205.2</v>
+        <v>1379</v>
       </c>
       <c r="D41" s="46" t="inlineStr">
         <is>
-          <t>ม.</t>
+          <t>ตร.ม.</t>
         </is>
       </c>
       <c r="E41" s="46" t="n">
-        <v>205.2</v>
+        <v>1379</v>
       </c>
       <c r="F41" s="46" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G41" s="47" t="inlineStr">
         <is>
@@ -10935,23 +11133,23 @@
       </c>
       <c r="H41" s="46" t="inlineStr">
         <is>
-          <t>โมเดล คานทับหลัง</t>
+          <t>โมเดล</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="46" t="inlineStr">
         <is>
-          <t>3.2.4</t>
+          <t>3.1.7</t>
         </is>
       </c>
       <c r="B42" s="46" t="inlineStr">
         <is>
-          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังวงกบประตู +2.60 (คอนกรีต ไม้แบบ)</t>
+          <t>ตะแกรงกันนก/ช่องระบายอากาศ ระดับ +4.50 ถึง +5.20 รอบอาคาร</t>
         </is>
       </c>
       <c r="C42" s="46" t="n">
-        <v>205.2</v>
+        <v>216</v>
       </c>
       <c r="D42" s="46" t="inlineStr">
         <is>
@@ -10959,10 +11157,10 @@
         </is>
       </c>
       <c r="E42" s="46" t="n">
-        <v>205.2</v>
+        <v>216</v>
       </c>
       <c r="F42" s="46" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G42" s="47" t="inlineStr">
         <is>
@@ -10971,34 +11169,34 @@
       </c>
       <c r="H42" s="46" t="inlineStr">
         <is>
-          <t>โมเดล คานเอ็น</t>
+          <t>เส้นรอบอาคาร - ประตูม้วน</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="46" t="inlineStr">
         <is>
-          <t>3.2.5</t>
+          <t>3.2.1</t>
         </is>
       </c>
       <c r="B43" s="46" t="inlineStr">
         <is>
-          <t>เสาเอ็น คสล. 0.15x0.10 ม. สูง 3.85 ม. (กลางช่วงเสา 6 ม. และข้างวงกบประตู)</t>
+          <t>ผนังก่ออิฐมวลเบา หนา 0.15 ม. +0.50 ถึง +4.35 (ต่ำกว่าหัวเสา คสล. 0.15 ม.)</t>
         </is>
       </c>
       <c r="C43" s="46" t="n">
-        <v>38</v>
+        <v>750.67</v>
       </c>
       <c r="D43" s="46" t="inlineStr">
         <is>
-          <t>ต้น</t>
+          <t>ตร.ม.</t>
         </is>
       </c>
       <c r="E43" s="46" t="n">
-        <v>38</v>
+        <v>744.63</v>
       </c>
       <c r="F43" s="46" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G43" s="47" t="inlineStr">
         <is>
@@ -11007,34 +11205,34 @@
       </c>
       <c r="H43" s="46" t="inlineStr">
         <is>
-          <t>โมเดล เสาเอ็น</t>
+          <t>โมเดล (ผนัง W1 หักเสาเอ็น/คานเอ็น/ประตู)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="46" t="inlineStr">
         <is>
-          <t>3.3.1</t>
+          <t>3.2.3</t>
         </is>
       </c>
       <c r="B44" s="46" t="inlineStr">
         <is>
-          <t>พื้นขัดมันผสม Floor Hardener</t>
+          <t>คานทับหลัง คสล. 0.15x0.15 ม. ระดับ +4.35 ถึง +4.50 (คอนกรีต ไม้แบบ)</t>
         </is>
       </c>
       <c r="C44" s="46" t="n">
-        <v>3206.48</v>
+        <v>205.2</v>
       </c>
       <c r="D44" s="46" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
+          <t>ม.</t>
         </is>
       </c>
       <c r="E44" s="46" t="n">
-        <v>3206.48</v>
+        <v>205.2</v>
       </c>
       <c r="F44" s="46" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G44" s="47" t="inlineStr">
         <is>
@@ -11043,95 +11241,95 @@
       </c>
       <c r="H44" s="46" t="inlineStr">
         <is>
-          <t>ตาราง S6.1</t>
+          <t>โมเดล คานทับหลัง</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="46" t="inlineStr">
         <is>
-          <t>4.1.1</t>
+          <t>3.2.4</t>
         </is>
       </c>
       <c r="B45" s="46" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับพื้นถนนรอบอาคาร (I22-22) รวมค่าตอก</t>
+          <t>คานเอ็น คสล. 0.15x0.10 ม. ระดับหลังวงกบประตู +2.60 (คอนกรีต ไม้แบบ)</t>
         </is>
       </c>
       <c r="C45" s="46" t="n">
-        <v>249</v>
+        <v>205.2</v>
       </c>
       <c r="D45" s="46" t="inlineStr">
         <is>
-          <t>ต้น</t>
+          <t>ม.</t>
         </is>
       </c>
       <c r="E45" s="46" t="n">
-        <v>232</v>
+        <v>205.2</v>
       </c>
       <c r="F45" s="46" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="G45" s="48" t="inlineStr">
-        <is>
-          <t>ต่าง – ตรวจ</t>
+        <v>-0</v>
+      </c>
+      <c r="G45" s="47" t="inlineStr">
+        <is>
+          <t>ตรง</t>
         </is>
       </c>
       <c r="H45" s="46" t="inlineStr">
         <is>
-          <t>ผัง S201 (ตาราง S2 = 249)</t>
+          <t>โมเดล คานเอ็น</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="46" t="inlineStr">
         <is>
-          <t>4.1.2</t>
+          <t>3.2.5</t>
         </is>
       </c>
       <c r="B46" s="46" t="inlineStr">
         <is>
-          <t>ฐาน F1A 0.60x0.60x0.30 ม. รับพื้นถนน</t>
+          <t>เสาเอ็น คสล. 0.15x0.10 ม. สูง 3.85 ม. (กลางช่วงเสา 6 ม. และข้างวงกบประตู)</t>
         </is>
       </c>
       <c r="C46" s="46" t="n">
-        <v>249</v>
+        <v>38</v>
       </c>
       <c r="D46" s="46" t="inlineStr">
         <is>
-          <t>ฐาน</t>
+          <t>ต้น</t>
         </is>
       </c>
       <c r="E46" s="46" t="n">
-        <v>232</v>
+        <v>38</v>
       </c>
       <c r="F46" s="46" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="G46" s="48" t="inlineStr">
-        <is>
-          <t>ต่าง – ตรวจ</t>
+        <v>0</v>
+      </c>
+      <c r="G46" s="47" t="inlineStr">
+        <is>
+          <t>ตรง</t>
         </is>
       </c>
       <c r="H46" s="46" t="inlineStr">
         <is>
-          <t>ผัง S201 (ตาราง S1.1 = 249)</t>
+          <t>โมเดล เสาเอ็น</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="46" t="inlineStr">
         <is>
-          <t>4.1.3</t>
+          <t>3.3.1</t>
         </is>
       </c>
       <c r="B47" s="46" t="inlineStr">
         <is>
-          <t>พื้นถนน S2 คสล. หนา 0.15 ม. TOP ±0.00 พร้อมรอยต่อ/ตัดรอยต่อ</t>
+          <t>พื้นขัดมันผสม Floor Hardener</t>
         </is>
       </c>
       <c r="C47" s="46" t="n">
-        <v>2440.69</v>
+        <v>3206.48</v>
       </c>
       <c r="D47" s="46" t="inlineStr">
         <is>
@@ -11139,151 +11337,151 @@
         </is>
       </c>
       <c r="E47" s="46" t="n">
-        <v>2384.78</v>
+        <v>3206.48</v>
       </c>
       <c r="F47" s="46" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="G47" s="48" t="inlineStr">
-        <is>
-          <t>ใกล้เคียง (≤5%)</t>
+        <v>0</v>
+      </c>
+      <c r="G47" s="47" t="inlineStr">
+        <is>
+          <t>ตรง</t>
         </is>
       </c>
       <c r="H47" s="46" t="inlineStr">
         <is>
-          <t>โมเดล (แนวเขต S202 หักอาคาร/ถัง/ทางลาด)</t>
+          <t>ตาราง S6.1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="46" t="inlineStr">
         <is>
-          <t>4.1.4</t>
+          <t>4.1.1</t>
         </is>
       </c>
       <c r="B48" s="46" t="inlineStr">
         <is>
-          <t>พื้น AF01 / SF02 ระดับถนน</t>
+          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับพื้นถนนรอบอาคาร (I22-22) รวมค่าตอก</t>
         </is>
       </c>
       <c r="C48" s="46" t="n">
-        <v>110.14</v>
+        <v>249</v>
       </c>
       <c r="D48" s="46" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
+          <t>ต้น</t>
         </is>
       </c>
       <c r="E48" s="46" t="n">
-        <v>110.14</v>
+        <v>232</v>
       </c>
       <c r="F48" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="47" t="inlineStr">
-        <is>
-          <t>ตรง</t>
+        <v>7.3</v>
+      </c>
+      <c r="G48" s="48" t="inlineStr">
+        <is>
+          <t>ต่าง – ตรวจ</t>
         </is>
       </c>
       <c r="H48" s="46" t="inlineStr">
         <is>
-          <t>ตาราง S6.1</t>
+          <t>ผัง S201 (ตาราง S2 = 249)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="46" t="inlineStr">
         <is>
-          <t>4.1.5</t>
+          <t>4.1.2</t>
         </is>
       </c>
       <c r="B49" s="46" t="inlineStr">
         <is>
-          <t>ทราย/หินคลุกรองใต้พื้นถนน S2 หนา 0.10 ม. บดอัด</t>
+          <t>ฐาน F1A 0.60x0.60x0.30 ม. รับพื้นถนน</t>
         </is>
       </c>
       <c r="C49" s="46" t="n">
-        <v>244.07</v>
+        <v>249</v>
       </c>
       <c r="D49" s="46" t="inlineStr">
         <is>
-          <t>ลบ.ม.</t>
+          <t>ฐาน</t>
         </is>
       </c>
       <c r="E49" s="46" t="n">
-        <v>244.07</v>
+        <v>232</v>
       </c>
       <c r="F49" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="47" t="inlineStr">
-        <is>
-          <t>ตรง</t>
+        <v>7.3</v>
+      </c>
+      <c r="G49" s="48" t="inlineStr">
+        <is>
+          <t>ต่าง – ตรวจ</t>
         </is>
       </c>
       <c r="H49" s="46" t="inlineStr">
         <is>
-          <t>S2 x 0.10</t>
+          <t>ผัง S201 (ตาราง S1.1 = 249)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="46" t="inlineStr">
         <is>
-          <t>4.3.1</t>
+          <t>4.1.3</t>
         </is>
       </c>
       <c r="B50" s="46" t="inlineStr">
         <is>
-          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
+          <t>พื้นถนน S2 คสล. หนา 0.15 ม. TOP ±0.00 พร้อมรอยต่อ/ตัดรอยต่อ</t>
         </is>
       </c>
       <c r="C50" s="46" t="n">
-        <v>6</v>
+        <v>2440.69</v>
       </c>
       <c r="D50" s="46" t="inlineStr">
         <is>
-          <t>ต้น</t>
+          <t>ตร.ม.</t>
         </is>
       </c>
       <c r="E50" s="46" t="n">
-        <v>6</v>
+        <v>2384.78</v>
       </c>
       <c r="F50" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="47" t="inlineStr">
-        <is>
-          <t>ตรง</t>
+        <v>2.3</v>
+      </c>
+      <c r="G50" s="48" t="inlineStr">
+        <is>
+          <t>ใกล้เคียง (≤5%)</t>
         </is>
       </c>
       <c r="H50" s="46" t="inlineStr">
         <is>
-          <t>ผัง S201</t>
+          <t>โมเดล (แนวเขต S202 หักอาคาร/ถัง/ทางลาด)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="46" t="inlineStr">
         <is>
-          <t>4.4.1</t>
+          <t>4.1.4</t>
         </is>
       </c>
       <c r="B51" s="46" t="inlineStr">
         <is>
-          <t>ขุดดินถังเก็บน้ำใต้ดิน ~12.12 x 6.63 ม. ลึก 3.00 ม. และขนทิ้ง</t>
+          <t>พื้น AF01 / SF02 ระดับถนน</t>
         </is>
       </c>
       <c r="C51" s="46" t="n">
-        <v>241.07</v>
+        <v>110.14</v>
       </c>
       <c r="D51" s="46" t="inlineStr">
         <is>
-          <t>ลบ.ม.</t>
+          <t>ตร.ม.</t>
         </is>
       </c>
       <c r="E51" s="46" t="n">
-        <v>241.07</v>
+        <v>110.14</v>
       </c>
       <c r="F51" s="46" t="n">
         <v>0</v>
@@ -11295,31 +11493,31 @@
       </c>
       <c r="H51" s="46" t="inlineStr">
         <is>
-          <t>ขนาดถังจากเวกเตอร์</t>
+          <t>ตาราง S6.1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="46" t="inlineStr">
         <is>
-          <t>4.4.2</t>
+          <t>4.1.5</t>
         </is>
       </c>
       <c r="B52" s="46" t="inlineStr">
         <is>
-          <t>พื้นถังเก็บน้ำใต้ดิน คสล. หนา 0.25 ม. (TF -2.60 / BF -2.85) พร้อมคอนกรีตหยาบ/ทราย</t>
+          <t>ทราย/หินคลุกรองใต้พื้นถนน S2 หนา 0.10 ม. บดอัด</t>
         </is>
       </c>
       <c r="C52" s="46" t="n">
-        <v>80.36</v>
+        <v>244.07</v>
       </c>
       <c r="D52" s="46" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
+          <t>ลบ.ม.</t>
         </is>
       </c>
       <c r="E52" s="46" t="n">
-        <v>80.36</v>
+        <v>244.07</v>
       </c>
       <c r="F52" s="46" t="n">
         <v>0</v>
@@ -11331,34 +11529,34 @@
       </c>
       <c r="H52" s="46" t="inlineStr">
         <is>
-          <t>ขนาดถังจากเวกเตอร์</t>
+          <t>S2 x 0.10</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="46" t="inlineStr">
         <is>
-          <t>4.5.1</t>
+          <t>4.3.1</t>
         </is>
       </c>
       <c r="B53" s="46" t="inlineStr">
         <is>
-          <t>รางระบายน้ำ คสล. พร้อมฝาปิด ตามแนวเขตที่ดิน</t>
+          <t>เสาเข็มตอก I-220x220 ยาว 22 ม. รับฐานหม้อแปลง (I22-TR) รวมค่าตอก</t>
         </is>
       </c>
       <c r="C53" s="46" t="n">
-        <v>302</v>
+        <v>6</v>
       </c>
       <c r="D53" s="46" t="inlineStr">
         <is>
-          <t>ม.</t>
+          <t>ต้น</t>
         </is>
       </c>
       <c r="E53" s="46" t="n">
-        <v>300.09</v>
+        <v>6</v>
       </c>
       <c r="F53" s="46" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="G53" s="47" t="inlineStr">
         <is>
@@ -11367,31 +11565,31 @@
       </c>
       <c r="H53" s="46" t="inlineStr">
         <is>
-          <t>โมเดล (แนวราง)</t>
+          <t>ผัง S201</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="46" t="inlineStr">
         <is>
-          <t>4.5.3</t>
+          <t>4.4.1</t>
         </is>
       </c>
       <c r="B54" s="46" t="inlineStr">
         <is>
-          <t>ท่อระบายน้ำฝนใต้ดิน PVC Ø4" จากท่อลงถึงรางระบายน้ำ</t>
+          <t>ขุดดินถังเก็บน้ำใต้ดิน ~12.12 x 6.63 ม. ลึก 3.00 ม. และขนทิ้ง</t>
         </is>
       </c>
       <c r="C54" s="46" t="n">
-        <v>10</v>
+        <v>241.07</v>
       </c>
       <c r="D54" s="46" t="inlineStr">
         <is>
-          <t>จุด</t>
+          <t>ลบ.ม.</t>
         </is>
       </c>
       <c r="E54" s="46" t="n">
-        <v>10</v>
+        <v>241.07</v>
       </c>
       <c r="F54" s="46" t="n">
         <v>0</v>
@@ -11403,31 +11601,31 @@
       </c>
       <c r="H54" s="46" t="inlineStr">
         <is>
-          <t>โมเดล</t>
+          <t>ขนาดถังจากเวกเตอร์</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="46" t="inlineStr">
         <is>
-          <t>4.6.1</t>
+          <t>4.4.2</t>
         </is>
       </c>
       <c r="B55" s="46" t="inlineStr">
         <is>
-          <t>เสาเข็ม I-260x260 + ฐาน 0.66x0.66 ม. แนวเขตที่ดินด้านใต้และตะวันออก (ไม่มีใน BOQ/ตาราง S2)</t>
+          <t>พื้นถังเก็บน้ำใต้ดิน คสล. หนา 0.25 ม. (TF -2.60 / BF -2.85) พร้อมคอนกรีตหยาบ/ทราย</t>
         </is>
       </c>
       <c r="C55" s="46" t="n">
-        <v>16</v>
+        <v>80.36</v>
       </c>
       <c r="D55" s="46" t="inlineStr">
         <is>
-          <t>ชุด</t>
+          <t>ตร.ม.</t>
         </is>
       </c>
       <c r="E55" s="46" t="n">
-        <v>16</v>
+        <v>80.36</v>
       </c>
       <c r="F55" s="46" t="n">
         <v>0</v>
@@ -11439,55 +11637,121 @@
       </c>
       <c r="H55" s="46" t="inlineStr">
         <is>
+          <t>ขนาดถังจากเวกเตอร์</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="46" t="inlineStr">
+        <is>
+          <t>4.5.1</t>
+        </is>
+      </c>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>รางระบายน้ำ คสล. พร้อมฝาปิด ตามแนวเขตที่ดิน</t>
+        </is>
+      </c>
+      <c r="C56" s="46" t="n">
+        <v>302</v>
+      </c>
+      <c r="D56" s="46" t="inlineStr">
+        <is>
+          <t>ม.</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="n">
+        <v>300.09</v>
+      </c>
+      <c r="F56" s="46" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G56" s="47" t="inlineStr">
+        <is>
+          <t>ตรง</t>
+        </is>
+      </c>
+      <c r="H56" s="46" t="inlineStr">
+        <is>
+          <t>โมเดล (แนวราง)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="46" t="inlineStr">
+        <is>
+          <t>4.5.3</t>
+        </is>
+      </c>
+      <c r="B57" s="46" t="inlineStr">
+        <is>
+          <t>ท่อระบายน้ำฝนใต้ดิน PVC Ø4" จากท่อลงถึงรางระบายน้ำ</t>
+        </is>
+      </c>
+      <c r="C57" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="D57" s="46" t="inlineStr">
+        <is>
+          <t>จุด</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="F57" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="47" t="inlineStr">
+        <is>
+          <t>ตรง</t>
+        </is>
+      </c>
+      <c r="H57" s="46" t="inlineStr">
+        <is>
+          <t>โมเดล</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="46" t="inlineStr">
+        <is>
+          <t>4.6.1</t>
+        </is>
+      </c>
+      <c r="B58" s="46" t="inlineStr">
+        <is>
+          <t>เสาเข็ม I-260x260 + ฐาน 0.66x0.66 ม. แนวเขตที่ดินด้านใต้และตะวันออก (ไม่มีใน BOQ/ตาราง S2)</t>
+        </is>
+      </c>
+      <c r="C58" s="46" t="n">
+        <v>16</v>
+      </c>
+      <c r="D58" s="46" t="inlineStr">
+        <is>
+          <t>ชุด</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="n">
+        <v>16</v>
+      </c>
+      <c r="F58" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="47" t="inlineStr">
+        <is>
+          <t>ตรง</t>
+        </is>
+      </c>
+      <c r="H58" s="46" t="inlineStr">
+        <is>
           <t>ผัง S201</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="46" t="n"/>
-      <c r="B56" s="46" t="n"/>
-      <c r="C56" s="46" t="n"/>
-      <c r="D56" s="46" t="n"/>
-      <c r="E56" s="46" t="n"/>
-      <c r="F56" s="46" t="n"/>
-      <c r="G56" s="46" t="n"/>
-      <c r="H56" s="46" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="46" t="inlineStr"/>
-      <c r="B57" s="41" t="inlineStr">
-        <is>
-          <t>สรุปประเด็นที่ต้องตรวจ</t>
-        </is>
-      </c>
-      <c r="C57" s="46" t="n"/>
-      <c r="D57" s="46" t="n"/>
-      <c r="E57" s="46" t="n"/>
-      <c r="F57" s="46" t="n"/>
-      <c r="G57" s="46" t="n"/>
-      <c r="H57" s="46" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="46" t="inlineStr"/>
-      <c r="B58" s="46" t="inlineStr">
-        <is>
-          <t>2.3.5: BOQ 40.45 เทียบ 38.87 (+4.1%) – โมเดล (แนวคาน B3 จาก S202) → ใช้ตาราง S3 (ความยาวรวมช่วงที่ซ้อนเสา) โมเดลวัดระหว่างผิวเสา – ยอมรับ</t>
-        </is>
-      </c>
-      <c r="C58" s="46" t="n"/>
-      <c r="D58" s="46" t="n"/>
-      <c r="E58" s="46" t="n"/>
-      <c r="F58" s="46" t="n"/>
-      <c r="G58" s="46" t="n"/>
-      <c r="H58" s="46" t="n"/>
-    </row>
     <row r="59">
-      <c r="A59" s="46" t="inlineStr"/>
-      <c r="B59" s="46" t="inlineStr">
-        <is>
-          <t>4.1.1: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S2 = 249) → ผู้ว่าจ้างยืนยัน 249 – ผังแสดง 232 ตำแหน่ง ขอตำแหน่ง 17 ต้นจากผู้ออกแบบ</t>
-        </is>
-      </c>
+      <c r="A59" s="46" t="n"/>
+      <c r="B59" s="46" t="n"/>
       <c r="C59" s="46" t="n"/>
       <c r="D59" s="46" t="n"/>
       <c r="E59" s="46" t="n"/>
@@ -11497,9 +11761,9 @@
     </row>
     <row r="60">
       <c r="A60" s="46" t="inlineStr"/>
-      <c r="B60" s="46" t="inlineStr">
-        <is>
-          <t>4.1.2: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S1.1 = 249) → ตาม 4.1.1 – ยอมรับ</t>
+      <c r="B60" s="41" t="inlineStr">
+        <is>
+          <t>สรุปประเด็นที่ต้องตรวจ</t>
         </is>
       </c>
       <c r="C60" s="46" t="n"/>
@@ -11513,7 +11777,7 @@
       <c r="A61" s="46" t="inlineStr"/>
       <c r="B61" s="46" t="inlineStr">
         <is>
-          <t>4.1.3: BOQ 2,440.69 เทียบ 2,384.78 (+2.3%) – โมเดล (แนวเขต S202 หักอาคาร/ถัง/ทางลาด) → ใช้ตาราง S6.1 (ค่าออกแบบ) โมเดลใช้แนวเขตที่ดินร่นเข้า 0.6 ม. โดยประมาณ – ยอมรับ</t>
+          <t>2.3.5: BOQ 40.45 เทียบ 38.87 (+4.1%) – โมเดล (แนวคาน B3 จาก S202) → ใช้ตาราง S3 (ความยาวรวมช่วงที่ซ้อนเสา) โมเดลวัดระหว่างผิวเสา – ยอมรับ</t>
         </is>
       </c>
       <c r="C61" s="46" t="n"/>
@@ -11523,6 +11787,48 @@
       <c r="G61" s="46" t="n"/>
       <c r="H61" s="46" t="n"/>
     </row>
+    <row r="62">
+      <c r="A62" s="46" t="inlineStr"/>
+      <c r="B62" s="46" t="inlineStr">
+        <is>
+          <t>4.1.1: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S2 = 249) → ผู้ว่าจ้างยืนยัน 249 – ผังแสดง 232 ตำแหน่ง ขอตำแหน่ง 17 ต้นจากผู้ออกแบบ</t>
+        </is>
+      </c>
+      <c r="C62" s="46" t="n"/>
+      <c r="D62" s="46" t="n"/>
+      <c r="E62" s="46" t="n"/>
+      <c r="F62" s="46" t="n"/>
+      <c r="G62" s="46" t="n"/>
+      <c r="H62" s="46" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="46" t="inlineStr"/>
+      <c r="B63" s="46" t="inlineStr">
+        <is>
+          <t>4.1.2: BOQ 249.00 เทียบ 232.00 (+7.3%) – ผัง S201 (ตาราง S1.1 = 249) → ตาม 4.1.1 – ยอมรับ</t>
+        </is>
+      </c>
+      <c r="C63" s="46" t="n"/>
+      <c r="D63" s="46" t="n"/>
+      <c r="E63" s="46" t="n"/>
+      <c r="F63" s="46" t="n"/>
+      <c r="G63" s="46" t="n"/>
+      <c r="H63" s="46" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="46" t="inlineStr"/>
+      <c r="B64" s="46" t="inlineStr">
+        <is>
+          <t>4.1.3: BOQ 2,440.69 เทียบ 2,384.78 (+2.3%) – โมเดล (แนวเขต S202 หักอาคาร/ถัง/ทางลาด) → ใช้ตาราง S6.1 (ค่าออกแบบ) โมเดลใช้แนวเขตที่ดินร่นเข้า 0.6 ม. โดยประมาณ – ยอมรับ</t>
+        </is>
+      </c>
+      <c r="C64" s="46" t="n"/>
+      <c r="D64" s="46" t="n"/>
+      <c r="E64" s="46" t="n"/>
+      <c r="F64" s="46" t="n"/>
+      <c r="G64" s="46" t="n"/>
+      <c r="H64" s="46" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>